<commit_message>
Organization: refreshed requirements file
</commit_message>
<xml_diff>
--- a/input/requirements/Organization.xlsx
+++ b/input/requirements/Organization.xlsx
@@ -1,24 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30215"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Organization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="349" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{793ACCA0-2929-4BBD-A432-D6FA7DCE717A}"/>
+  <xr:revisionPtr revIDLastSave="668" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE04BCF3-BF31-4511-8967-42B0CF5ACD00}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="21120" tabRatio="553" firstSheet="2" activeTab="1" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="553" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
     <sheet name="Concept" sheetId="2" r:id="rId2"/>
-    <sheet name="Informatiebehoefte" sheetId="1" r:id="rId3"/>
-    <sheet name="Ongedekte informatiebehoefte" sheetId="3" r:id="rId4"/>
-    <sheet name="Overwegingen voor de toekomst" sheetId="4" r:id="rId5"/>
-    <sheet name="Ter discussie" sheetId="6" r:id="rId6"/>
+    <sheet name="Bronnen" sheetId="7" r:id="rId3"/>
+    <sheet name="Informatiebehoefte" sheetId="1" r:id="rId4"/>
+    <sheet name="Ongedekte informatiebehoefte" sheetId="3" r:id="rId5"/>
+    <sheet name="Overwegingen voor de toekomst" sheetId="4" r:id="rId6"/>
+    <sheet name="Ter discussie" sheetId="6" r:id="rId7"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="105" uniqueCount="85">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="142">
   <si>
     <t>Veld</t>
   </si>
@@ -52,13 +53,13 @@
     <t>Conceptbeschrijving</t>
   </si>
   <si>
-    <t>A formally or informally recognized grouping of people or organizations formed for the purpose of achieving some form of collective action.</t>
+    <t>Een formeel of informeel erkende groep van personen of organisaties die is opgericht met het doel een of andere vorm van collectieve actie te ondernemen.</t>
   </si>
   <si>
     <t>Doel</t>
   </si>
   <si>
-    <t xml:space="preserve">The organization may be used in a shared registry of contact and other information for various organizations or it can be used merely as a support for other resources that need to reference organizations, perhaps as a document, message or as a contained resource. </t>
+    <t>De organisatie kan worden opgenomen in een gezamenlijk register met contactgegevens en andere informatie voor diverse organisaties, of kan louter dienen als ondersteuning voor andere bronnen die naar organisaties moeten verwijzen, bijvoorbeeld in de vorm van een document, een bericht of een bijgevoegde FHIR-resource.</t>
   </si>
   <si>
     <t>Gebruiksscenario(’s)</t>
@@ -70,44 +71,113 @@
     <t>Representatie</t>
   </si>
   <si>
-    <t>[Beschrijf hier wat er voor de dossiervorming belangrijk is rondom de levenscyclus en instantiaties van het concept.]</t>
+    <t>x</t>
   </si>
   <si>
     <t>Alias(sen)</t>
   </si>
   <si>
-    <t>x</t>
+    <t>Verzekeraar, Afdeling, Zorgorganisatie</t>
   </si>
   <si>
     <t>Juist gebruik</t>
   </si>
   <si>
-    <t>Gebruikt voor het vastleggen van de informatie van de koepelorganisatie (Zorgorganisatie, verzekeraar etc.)
-companies
-institutions
-corporations
-departments
-community groups
-healthcare practice groups
-payer/insurer</t>
+    <t>Bijvoorbeeld:
+bedrijven
+instellingen
+ondernemingen
+afdelingen
+buurtgroepen
+groepen van zorgverleners
+betalers/verzekeraars</t>
   </si>
   <si>
     <t>Onjuist gebruik</t>
   </si>
   <si>
-    <t>Niet gebruikt  voor vastleggen van specifieke locaties van zorgorganisaties</t>
+    <t>Niet gebruikt  voor vastleggen van specifieke (fysieke) locaties van zorgorganisaties</t>
   </si>
   <si>
     <t>Referenties</t>
   </si>
   <si>
-    <t>[Relevante bronstandaarden of informatiebronnen die het ontwerp en de scope van het concept hebben beïnvloed.]</t>
+    <t>Zie tabblad Bronnen</t>
   </si>
   <si>
     <t>ART-DECOR-id</t>
   </si>
   <si>
-    <t>2.16.840.1.113883.2.4.3.11.60.153.1.7</t>
+    <t>2.16.840.1.113883.2.4.3.11.60.153.4.20/2026-06-24T00:00:00</t>
+  </si>
+  <si>
+    <t>type bron</t>
+  </si>
+  <si>
+    <t>link</t>
+  </si>
+  <si>
+    <t>aantekeningen</t>
+  </si>
+  <si>
+    <t>zibs.nl</t>
+  </si>
+  <si>
+    <t>https://zibs.nl/wiki/Zorgaanbieder-v3.4(2020NL)</t>
+  </si>
+  <si>
+    <t>openEHR</t>
+  </si>
+  <si>
+    <t>https://ckm.openehr.org/ckm/archetypes/1013.1.371/mindmap</t>
+  </si>
+  <si>
+    <t>FHIR R4 base</t>
+  </si>
+  <si>
+    <t>https://hl7.org/fhir/R4/organization.html</t>
+  </si>
+  <si>
+    <t>1.0.3-versie, heeft o.a. parent organisation en contactperson</t>
+  </si>
+  <si>
+    <t>zib-profiel</t>
+  </si>
+  <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/zibhealthcareproviderorganization</t>
+  </si>
+  <si>
+    <t>NL-core-R4</t>
+  </si>
+  <si>
+    <t>https://simplifier.net/nictiz-r4-zib2020/nlcorehealthcareproviderorganization</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM</t>
+  </si>
+  <si>
+    <t>https://www.xt-ehr.eu/fhir/models/en/StructureDefinition-EHDSOrganisation.html</t>
+  </si>
+  <si>
+    <t>EHDS FHIR</t>
+  </si>
+  <si>
+    <t>https://hl7.eu/fhir/base/StructureDefinition-organization-eu-core.html</t>
+  </si>
+  <si>
+    <t>mapping xt-EHR --&gt; FHIR</t>
+  </si>
+  <si>
+    <t>https://hl7.eu/fhir/base/map-ehdsorganisation.html</t>
+  </si>
+  <si>
+    <t>zib-issues</t>
+  </si>
+  <si>
+    <t>Spoedsamenvatting</t>
+  </si>
+  <si>
+    <t>https://decor.nictiz.nl/ad/#/acutezorg-/rules/templates/2.16.840.1.113883.2.4.3.11.60.66.10.77/2022-03-30T00:00:00</t>
   </si>
   <si>
     <t>Nummer</t>
@@ -134,10 +204,145 @@
     <t>Opmerkingen</t>
   </si>
   <si>
-    <t>[Nummer van de informatie-requirement start bij 1, sub behoeftes kunnen worden gemodelleerd met X.X of X.X.X]</t>
-  </si>
-  <si>
-    <t>[Naam waaraan de informatie-requirement te herkennen is]</t>
+    <t>ORG-001</t>
+  </si>
+  <si>
+    <t>Identifier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The organization’s identification number. </t>
+  </si>
+  <si>
+    <t>(identifier)</t>
+  </si>
+  <si>
+    <t>0..*</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM 1.0.0 Organization</t>
+  </si>
+  <si>
+    <t>ORG-002</t>
+  </si>
+  <si>
+    <t>(identifier)
+SHOULD For Dutch healthcare providers, the URA number or the AGB number is used, if possible.</t>
+  </si>
+  <si>
+    <t>Zib2020, Spoedsamenvatting, BgZ-MSZ</t>
+  </si>
+  <si>
+    <t>ORG-003</t>
+  </si>
+  <si>
+    <t>OrganizationType</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The type of healthcare provider, such as general hospital, or nursing home. </t>
+  </si>
+  <si>
+    <t>(coded; binding: extensible; codelist: selection of RoleCodeNL)</t>
+  </si>
+  <si>
+    <t>If this field is filled in and an AGB code is used for the HealthcareProviderIdentificationNumber, the type must match the type implicitly contained in the AGB code.</t>
+  </si>
+  <si>
+    <t>ORG-004</t>
+  </si>
+  <si>
+    <t>Type of organization, such as insurance company, healthcare provider etc.</t>
+  </si>
+  <si>
+    <t>Binding Description: (preferred): HL7 organisation_type</t>
+  </si>
+  <si>
+    <t>hl7:standardIndustryClassCode</t>
+  </si>
+  <si>
+    <t>OrganizationIndustryClass</t>
+  </si>
+  <si>
+    <t>0..1</t>
+  </si>
+  <si>
+    <t>ORG-005</t>
+  </si>
+  <si>
+    <t>OrganizationName</t>
+  </si>
+  <si>
+    <t>Name of the organization.</t>
+  </si>
+  <si>
+    <t>(string)</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM 1.0.0 Organization, BgZ-MSZ</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> If an identification number is given, the name must match the name that corresponds to the identification number.</t>
+  </si>
+  <si>
+    <t>Zie discussie</t>
+  </si>
+  <si>
+    <t>ORG-006</t>
+  </si>
+  <si>
+    <t>Contact.Address</t>
+  </si>
+  <si>
+    <t>An address for a contact within the organization</t>
+  </si>
+  <si>
+    <t>(ref. GBB-Address)
+SHALL An address of an organization can never be of use 'home'</t>
+  </si>
+  <si>
+    <t>Xt-EHR LIM 1.0.0 Organization, Spoedsamenvatting, BgZ MSZ</t>
+  </si>
+  <si>
+    <t>ORG-007</t>
+  </si>
+  <si>
+    <t>Contact.Telecom</t>
+  </si>
+  <si>
+    <t>Contact information to contact a person within the organization with.</t>
+  </si>
+  <si>
+    <t>(ref. GBB-ContactPoint)
+SHALL The telecom of an organization can never be of use 'home'</t>
+  </si>
+  <si>
+    <t>ORG-008</t>
+  </si>
+  <si>
+    <t>PartOf</t>
+  </si>
+  <si>
+    <t>(Reference to) The organization of which this organization forms a part. Needed to be able to track the hierarchy of organizations within an organization.</t>
+  </si>
+  <si>
+    <t>(ref. GBB-Organization)</t>
+  </si>
+  <si>
+    <t>0..1  If the resource is contained in another resource, it SHALL NOT contain nested Resources. e.g., a department in a hospital cannot be the target of another Organization.partOf</t>
+  </si>
+  <si>
+    <t>Actie</t>
+  </si>
+  <si>
+    <t>Notitie</t>
+  </si>
+  <si>
+    <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
+  </si>
+  <si>
+    <t>[Eventuele notitie]</t>
+  </si>
+  <si>
+    <t>[Naam van de informatie-requirement ]</t>
   </si>
   <si>
     <t>[Geef hier een tekstuele omschrijving van de behoefte die ingevuld wordt met de informatie-requirement]</t>
@@ -149,167 +354,137 @@
     <t>[Geef aan in welke situaties het element waarmee de informatie-requirement gedekt wordt er zou moeten zijn, en evt. wanneer het afwezig kan zijn]</t>
   </si>
   <si>
-    <t>[Geef aan of de informatie relevant is voor gebruik van het model voor zaken in het verleden, in het heden, en/of de toekomst. Vaak is slechts een van deze situaties in scope van het bouwblok, maar niet altijd]</t>
-  </si>
-  <si>
     <t>[Geef aan waar de behoefte vandaan komt, bv. een specifieke informatiestandaard of bepaalde zorgrichtlijn]</t>
   </si>
   <si>
-    <t>ORG-001</t>
-  </si>
-  <si>
-    <t>Identifier(+LocationNumber)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The organization’s identification number. </t>
-  </si>
-  <si>
-    <t>0..* For Dutch healthcare providers, the URA number or the AGB number is used, if possible. Depending on the context other ID's are also possible. For foreign or non-affiliated healthcare providers, another unique identification number can be used. This must be accompanied by the name and/or code of the issuing organization.</t>
-  </si>
-  <si>
-    <t>Zib2020</t>
-  </si>
-  <si>
-    <t>ORG-002</t>
+    <t>Data element</t>
+  </si>
+  <si>
+    <t>Informatiestandaard</t>
+  </si>
+  <si>
+    <t>Uitleg</t>
+  </si>
+  <si>
+    <t>Uitkomst</t>
+  </si>
+  <si>
+    <t>contact.name</t>
+  </si>
+  <si>
+    <t>FHIR R5</t>
+  </si>
+  <si>
+    <t>In de Xt-EHR komt dit niet voor, maar dit kan veel context toevoegen aan een contact</t>
+  </si>
+  <si>
+    <t>contact.purpose</t>
+  </si>
+  <si>
+    <t xml:space="preserve">In de Xt-EHR komt dit niet voor, maar dit kan veel context toevoegen aan een contact. Voorbeeld van een ziekenhuis https://www.ziekenhuisamstelland.nl/contact/ </t>
+  </si>
+  <si>
+    <t>organizationType</t>
+  </si>
+  <si>
+    <t>willen we de waardelijsten van zowel FHIR als zib houden?</t>
+  </si>
+  <si>
+    <t>Ter Discussie</t>
+  </si>
+  <si>
+    <t>zib2020</t>
+  </si>
+  <si>
+    <t xml:space="preserve">De container OrganizationLocation lijkt niet een fysieke locatie te duiden, maar te betekenen dat die instantiatie een onderdeel van een grotere organisatie is, en wel of niet een andere locatie heeft dan die grotere organisatie. </t>
+  </si>
+  <si>
+    <t>Organisatie en Locatie zijn uitgesplitst in 2 aparte GBB's. Vanuit Locatie wordt verwezen naar Organisatie. In Organisatie.PartOf is gekozen voor verwijzing naar Organisatie.</t>
   </si>
   <si>
     <t>DepartmentSpecialty</t>
   </si>
   <si>
-    <t xml:space="preserve">The specialty of the healthcare provider’s department. The departmental specialty can be filled in if further indication of the healthcare provider is needed. </t>
-  </si>
-  <si>
-    <t>0..* This refers to the recognized medical specialties as stated in the BIG Act.</t>
-  </si>
-  <si>
-    <t>Zie discussie</t>
-  </si>
-  <si>
-    <t>ORG-003</t>
-  </si>
-  <si>
-    <t>DepartmentType</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The type of healthcare provider, such as general hospital, or nursing home. </t>
-  </si>
-  <si>
-    <t>0..*</t>
-  </si>
-  <si>
-    <t>If this field is filled in and an AGB code is used for the HealthcareProviderIdentificationNumber, the type must match the type implicitly contained in the AGB code.</t>
-  </si>
-  <si>
-    <t>ORG-004</t>
-  </si>
-  <si>
-    <t>OrganizationName</t>
-  </si>
-  <si>
-    <t>Name of the organization. If an identification number is given, the name must match the name that corresponds to the identification number.</t>
-  </si>
-  <si>
-    <t>0..1</t>
-  </si>
-  <si>
-    <t>If an identification number is given, the name must match the name that corresponds to the identification number.</t>
-  </si>
-  <si>
-    <t>Xt-EHR LIM 1.0.0</t>
-  </si>
-  <si>
-    <t>ORG-005</t>
-  </si>
-  <si>
-    <t>Contact.Name</t>
-  </si>
-  <si>
-    <t>The name of the contact within the organization</t>
-  </si>
-  <si>
-    <t>ORG-006</t>
-  </si>
-  <si>
-    <t>Contact.Address</t>
-  </si>
-  <si>
-    <t>An address for a contact within the organization</t>
-  </si>
-  <si>
-    <t>An address of an organization can never be of use 'home'</t>
-  </si>
-  <si>
-    <t>ORG-007</t>
-  </si>
-  <si>
-    <t>Contact.Telecom</t>
-  </si>
-  <si>
-    <t>Contact information to contact a person within organization with</t>
-  </si>
-  <si>
-    <t xml:space="preserve">0..* </t>
-  </si>
-  <si>
-    <t>The telecom of an organization can never be of use 'home'</t>
-  </si>
-  <si>
-    <t>ORG-008</t>
-  </si>
-  <si>
-    <t>PartOf</t>
-  </si>
-  <si>
-    <t>The organization of which this organization forms a part. Needed to be able to track the hierarchy of organizations within an organization.</t>
-  </si>
-  <si>
-    <t>Actie</t>
-  </si>
-  <si>
-    <t>Notitie</t>
-  </si>
-  <si>
-    <t>[Actie om te ondernemen, kies uit de 3 acties: cluster, andere bouwsteen en modelleren]</t>
-  </si>
-  <si>
-    <t>[Eventuele notitie]</t>
-  </si>
-  <si>
-    <t>[Naam van de informatie-requirement ]</t>
-  </si>
-  <si>
-    <t>Ter Discussie</t>
-  </si>
-  <si>
-    <t>Data element</t>
-  </si>
-  <si>
-    <t>Informatiestandaard</t>
-  </si>
-  <si>
-    <t>Uitleg</t>
-  </si>
-  <si>
-    <t>Uitkomst</t>
-  </si>
-  <si>
-    <t>zib2020</t>
-  </si>
-  <si>
-    <t xml:space="preserve">De container OrganizationLocation lijkt niet een fysieke locatie te duiden, maar te betekenen dat die instantiatie een onderdeel van een grotere organisatie is, en wel of niet een andere locatie heeft dan die grotere organisatie. </t>
-  </si>
-  <si>
-    <t>Discussie over het gebruik van HealthCareServices (FHIR element) in de plaats. Handig voor declaraties. Staat ook als verwijzing in PractitionerRole</t>
+    <t>Discussie over het gebruik van HealthCareServices (FHIR element) in de plaats. Handig voor declaraties. Staat ook als verwijzing in PractitionerRole. Zie ook Zib issue: https://nictiz.atlassian.net/browse/ZIB-452</t>
+  </si>
+  <si>
+    <t>ZIB-2941 -&gt; verwijder DepartmentSpecialty (AfdelingSpecialisme) uit Organization</t>
+  </si>
+  <si>
+    <t>Waardelijst organisation_type</t>
   </si>
   <si>
     <t>Xt-EHR (preferred): HL7 organisation_type, Zib2020</t>
+  </si>
+  <si>
+    <t>Gewerkt met additional bindings, beide waardelijsten toegevoegd in FHIR profiel, HL7 organisation_type gewijzigd van example naar preferred.</t>
+  </si>
+  <si>
+    <t>LocationNumber</t>
+  </si>
+  <si>
+    <t>LocationNumber wordt gezien als identifier of naam. Hoe om te gaan met datatype integer tov identifier?</t>
+  </si>
+  <si>
+    <t>LocationNumber heeft geen mappingen. We zien het daarom niet als informatierequirement</t>
+  </si>
+  <si>
+    <t>Contact</t>
+  </si>
+  <si>
+    <t>Adres en telecom verbonden aan een Contact. Kardinaliteiten nog onduidelijk</t>
+  </si>
+  <si>
+    <t>Contact incl. kardinaliteiten als "pre-adopt" meegenomen uit R5; Elementen Telecom en Address komen in R5 niet meer los voor, maar slechts als onderdeel van Contact.</t>
+  </si>
+  <si>
+    <t>Na afstemming met leveranciers besloten om dit terug te draaien en Kard. 0..* aan te houden.</t>
+  </si>
+  <si>
+    <t>Obligation nog niet toegevoegd, discussie gaande</t>
+  </si>
+  <si>
+    <t>Zie "Overwegingen voor de toekomst"</t>
+  </si>
+  <si>
+    <t>ZIB-464</t>
+  </si>
+  <si>
+    <t>Wens voor splitsing Afdeling en Specialisme. Is dit een IB?</t>
+  </si>
+  <si>
+    <t>ZIB-2941 -&gt; verwijder uit Organization</t>
+  </si>
+  <si>
+    <t>Organization.name</t>
+  </si>
+  <si>
+    <t>SSV</t>
+  </si>
+  <si>
+    <t>In de SSV meerdere namen mogelijk, kardinaliteit 0..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat (in het FHIR profiel is .name 1..1)</t>
+  </si>
+  <si>
+    <t>Organization.name aankaarten bij FHIR EU, omdat deze 1..1 ipv de LIM die aangeeft dat deze 0..1 is.</t>
+  </si>
+  <si>
+    <t>Organization.Address</t>
+  </si>
+  <si>
+    <t>In de SSV meerdere adressen mogelijk, kardinaliteit 0..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat. Dit wordt opgelost als de modeleering vanuit R% teruggezet wordt naar R4 (zonder contact container)</t>
+  </si>
+  <si>
+    <t>Organization.Telecom</t>
+  </si>
+  <si>
+    <t>In de SSV meerdere Telecom mogelijk, kardinaliteit 0..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat. Dit wordt opgelost als de modeleering vanuit R% teruggezet wordt naar R4 (zonder contact container)</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="9">
+  <fonts count="15">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -376,16 +551,62 @@
       <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos"/>
+      <family val="2"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFE97132"/>
+        <bgColor rgb="FF000000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -404,11 +625,62 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </left>
+      <right/>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFF1A983"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFF1A983"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </right>
+      <top style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </top>
+      <bottom style="thin">
+        <color theme="5" tint="0.39997558519241921"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -439,12 +711,87 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="29">
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor indexed="64"/>
+          <bgColor auto="1"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
     <dxf>
       <font>
         <b val="0"/>
@@ -578,6 +925,173 @@
         </patternFill>
       </fill>
       <alignment textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="none"/>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="none">
+          <fgColor theme="5"/>
+          <bgColor theme="5"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment wrapText="1"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="none"/>
+      </font>
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color rgb="FFFFFFFF"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FF000000"/>
+          <bgColor rgb="FFE97132"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1287,13 +1801,67 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F34DEBB5-2EFB-4078-A24C-EE66E3791A2F}" name="Tabel1" displayName="Tabel1" ref="B3:E21" totalsRowShown="0" headerRowDxfId="5" dataDxfId="4">
-  <autoFilter ref="B3:E21" xr:uid="{F34DEBB5-2EFB-4078-A24C-EE66E3791A2F}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{59B5D8CA-526E-41E2-9015-923318959E98}" name="Tabel4" displayName="Tabel4" ref="A2:B11" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+  <autoFilter ref="A2:B11" xr:uid="{59B5D8CA-526E-41E2-9015-923318959E98}"/>
+  <tableColumns count="2">
+    <tableColumn id="1" xr3:uid="{50EFEBF6-4893-432E-BEA1-588A83D972CB}" name="Veld" dataDxfId="26"/>
+    <tableColumn id="2" xr3:uid="{9FB3B455-2F07-4EC4-A31C-65E3885F100A}" name="Beschrijving" dataDxfId="25"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AE4E70E2-B46F-4B62-81CF-884CAD44739D}" name="Tabel5" displayName="Tabel5" ref="A1:C11" totalsRowShown="0" headerRowDxfId="24">
+  <autoFilter ref="A1:C11" xr:uid="{AE4E70E2-B46F-4B62-81CF-884CAD44739D}"/>
+  <tableColumns count="3">
+    <tableColumn id="1" xr3:uid="{353B1C84-B074-472C-8FDA-BF6BED2D63C8}" name="type bron" dataDxfId="23"/>
+    <tableColumn id="2" xr3:uid="{0B17EAA3-957B-45FC-A6C7-6D847A216C50}" name="link" dataCellStyle="Hyperlink"/>
+    <tableColumn id="3" xr3:uid="{8B33B7A8-D1F0-4831-95B4-64521C7111E4}" name="aantekeningen"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}" name="Tabel2" displayName="Tabel2" ref="A2:H14" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+  <autoFilter ref="A2:H14" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}"/>
+  <tableColumns count="8">
+    <tableColumn id="1" xr3:uid="{AEDCF761-C41E-45F9-8585-F195D983B89C}" name="Nummer" dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{635CD206-F27E-4A6A-BC65-EEED36933D1E}" name="Naam" dataDxfId="19"/>
+    <tableColumn id="3" xr3:uid="{8EF3A9D6-055E-4CB8-96A3-6552DF1766C8}" name="Omschrijving" dataDxfId="18"/>
+    <tableColumn id="4" xr3:uid="{C3044835-AC84-438A-ADC2-CAD99CE92BD0}" name="Variabiliteit" dataDxfId="17"/>
+    <tableColumn id="5" xr3:uid="{AA18877F-FB5A-4805-A5CF-69206661B387}" name="Aanwezigheid" dataDxfId="16"/>
+    <tableColumn id="6" xr3:uid="{564C5C8F-5623-4C63-8144-810E58143EDA}" name="Verleden/heden/toekomst" dataDxfId="15"/>
+    <tableColumn id="7" xr3:uid="{58DBAFD8-EA1C-440F-9872-7271A13F1C90}" name="Herkomst" dataDxfId="14"/>
+    <tableColumn id="8" xr3:uid="{F805880C-4939-45E5-9047-13B213C612A8}" name="Opmerkingen" dataDxfId="13"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{E20A176F-3671-4755-B06A-A662E9E9670D}" name="Tabel6" displayName="Tabel6" ref="A2:D5" totalsRowShown="0" headerRowDxfId="12" dataDxfId="11">
+  <autoFilter ref="A2:D5" xr:uid="{E20A176F-3671-4755-B06A-A662E9E9670D}"/>
   <tableColumns count="4">
-    <tableColumn id="1" xr3:uid="{68B36AAD-2300-4CA0-AA10-5F1A41ABB17E}" name="Data element" dataDxfId="3"/>
-    <tableColumn id="2" xr3:uid="{341D4A74-791C-425D-B379-8FC69CAF6C79}" name="Informatiestandaard" dataDxfId="2"/>
-    <tableColumn id="3" xr3:uid="{79F7C4DD-833C-4C2D-936C-815F18189410}" name="Uitleg" dataDxfId="1"/>
-    <tableColumn id="4" xr3:uid="{D3C54DC8-E13B-4401-86E0-4E8753D268FA}" name="Uitkomst" dataDxfId="0"/>
+    <tableColumn id="1" xr3:uid="{3C3A3648-FA1B-4745-AA0F-56FD15B31549}" name="Data element" dataDxfId="10"/>
+    <tableColumn id="2" xr3:uid="{5AB75249-FC0C-4020-93EF-4E5B4F92C328}" name="Informatiestandaard" dataDxfId="9"/>
+    <tableColumn id="3" xr3:uid="{304BF3A6-44F1-48DF-87D2-1D29D19573B9}" name="Uitleg" dataDxfId="8"/>
+    <tableColumn id="4" xr3:uid="{F0B70321-80D5-49AC-89C4-9533F7F4B3BF}" name="Uitkomst" dataDxfId="7"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+</table>
+</file>
+
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{F34DEBB5-2EFB-4078-A24C-EE66E3791A2F}" name="Tabel1" displayName="Tabel1" ref="B3:F20" totalsRowShown="0" headerRowDxfId="6" dataDxfId="5">
+  <autoFilter ref="B3:F20" xr:uid="{F34DEBB5-2EFB-4078-A24C-EE66E3791A2F}"/>
+  <tableColumns count="5">
+    <tableColumn id="1" xr3:uid="{68B36AAD-2300-4CA0-AA10-5F1A41ABB17E}" name="Data element" dataDxfId="4"/>
+    <tableColumn id="2" xr3:uid="{341D4A74-791C-425D-B379-8FC69CAF6C79}" name="Informatiestandaard" dataDxfId="3"/>
+    <tableColumn id="3" xr3:uid="{79F7C4DD-833C-4C2D-936C-815F18189410}" name="Uitleg" dataDxfId="2"/>
+    <tableColumn id="4" xr3:uid="{D3C54DC8-E13B-4401-86E0-4E8753D268FA}" name="Uitkomst" dataDxfId="1"/>
+    <tableColumn id="5" xr3:uid="{47354D9D-ADCE-4E5D-995C-AEEFC62D7612}" name="Opmerkingen" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1617,7 +2185,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F1013F7-63B2-4F83-92B0-1C8153859891}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="218.42578125" customWidth="1"/>
   </cols>
@@ -1634,105 +2202,231 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2CC1E3B3-D087-4A2B-920B-9BA971FAD64B}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="23" customWidth="1"/>
-    <col min="2" max="2" width="29.140625" customWidth="1"/>
+    <col min="2" max="2" width="140.28515625" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" ht="190.5" customHeight="1">
       <c r="A1" s="3"/>
     </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:2" ht="15">
+      <c r="A2" s="21" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="21" t="s">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:2">
-      <c r="A3" t="s">
+    <row r="3" spans="1:2" ht="15">
+      <c r="A3" s="22" t="s">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="22" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:2">
-      <c r="A4" t="s">
+    <row r="4" spans="1:2" ht="43.5">
+      <c r="A4" s="22" t="s">
         <v>4</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B4" s="22" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="5" spans="1:2">
-      <c r="A5" t="s">
+    <row r="5" spans="1:2" ht="15">
+      <c r="A5" s="22" t="s">
         <v>6</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B5" s="22" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:2">
-      <c r="A6" t="s">
+    <row r="6" spans="1:2" ht="15">
+      <c r="A6" s="22" t="s">
         <v>8</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B6" s="22" t="s">
         <v>9</v>
       </c>
     </row>
-    <row r="7" spans="1:2">
-      <c r="A7" t="s">
+    <row r="7" spans="1:2" ht="15">
+      <c r="A7" s="22" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="3" t="s">
+      <c r="B7" s="22" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="8" spans="1:2" ht="174">
-      <c r="A8" t="s">
+    <row r="8" spans="1:2" ht="138.75" customHeight="1">
+      <c r="A8" s="22" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="3" t="s">
+      <c r="B8" s="22" t="s">
         <v>13</v>
       </c>
     </row>
-    <row r="9" spans="1:2">
-      <c r="A9" t="s">
+    <row r="9" spans="1:2" ht="15">
+      <c r="A9" s="22" t="s">
         <v>14</v>
       </c>
-      <c r="B9" t="s">
+      <c r="B9" s="22" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="10" spans="1:2">
-      <c r="A10" t="s">
+    <row r="10" spans="1:2" ht="15">
+      <c r="A10" s="22" t="s">
         <v>16</v>
       </c>
-      <c r="B10" t="s">
+      <c r="B10" s="22" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="11" spans="1:2">
-      <c r="A11" t="s">
+    <row r="11" spans="1:2" ht="15">
+      <c r="A11" s="22" t="s">
         <v>18</v>
       </c>
-      <c r="B11" t="s">
+      <c r="B11" s="23" t="s">
         <v>19</v>
       </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E4656AF1-42FD-4E84-8EE1-8568D7C6AEE8}">
+  <dimension ref="A1:C12"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="23.5703125" customWidth="1"/>
+    <col min="2" max="2" width="106.28515625" customWidth="1"/>
+    <col min="3" max="3" width="62.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3">
+      <c r="A1" s="12" t="s">
+        <v>20</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>21</v>
+      </c>
+      <c r="C1" s="12" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="15">
+      <c r="A2" s="13" t="s">
+        <v>23</v>
+      </c>
+      <c r="B2" s="14" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="29.25">
+      <c r="A3" s="13" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" s="14" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="15">
+      <c r="A4" s="13" t="s">
+        <v>27</v>
+      </c>
+      <c r="B4" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="C4" s="24" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="29.25">
+      <c r="A5" s="13" t="s">
+        <v>30</v>
+      </c>
+      <c r="B5" s="14" t="s">
+        <v>31</v>
+      </c>
+      <c r="C5" s="16"/>
+    </row>
+    <row r="6" spans="1:3" ht="29.25">
+      <c r="A6" s="13" t="s">
+        <v>32</v>
+      </c>
+      <c r="B6" s="14" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="28.9">
+      <c r="A7" s="13" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" s="15" t="s">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="28.9">
+      <c r="A8" s="13" t="s">
+        <v>36</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="43.15">
+      <c r="A9" s="13" t="s">
+        <v>38</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="28.9">
+      <c r="A10" s="13" t="s">
+        <v>40</v>
+      </c>
+      <c r="B10" s="14"/>
+    </row>
+    <row r="11" spans="1:3" ht="15">
+      <c r="A11" t="s">
+        <v>41</v>
+      </c>
+      <c r="B11" s="15" t="s">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="15"/>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B4" r:id="rId1" xr:uid="{C7D966CA-C6CB-4183-BBA3-54EA1ABF8AEE}"/>
+    <hyperlink ref="B6" r:id="rId2" xr:uid="{714DC51B-F00F-4956-B2FD-68C8B6E5BE15}"/>
+    <hyperlink ref="B5" r:id="rId3" xr:uid="{C9FF6A25-B16C-455F-997B-799DC66A9421}"/>
+    <hyperlink ref="B7" r:id="rId4" xr:uid="{7537026A-3648-43A4-85B1-4D41007BC509}"/>
+    <hyperlink ref="B8" r:id="rId5" xr:uid="{8ECA5E5A-7DB0-4A42-AFB0-1A65D87AC5C9}"/>
+    <hyperlink ref="B9" r:id="rId6" xr:uid="{5D12AB18-C915-444A-BF83-F1C3EFFEB15F}"/>
+    <hyperlink ref="B2" r:id="rId7" xr:uid="{243AB532-E225-406E-8344-C49AC95EE8F3}"/>
+    <hyperlink ref="B3" r:id="rId8" xr:uid="{A074D791-C70A-41DB-89D7-F2FBD624768F}"/>
+    <hyperlink ref="B11" r:id="rId9" location="/acutezorg-/rules/templates/2.16.840.1.113883.2.4.3.11.60.66.10.77/2022-03-30T00:00:00" xr:uid="{EC237B1A-B0CB-4576-8BF8-B8BF1D9CC33C}"/>
+  </hyperlinks>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <tableParts count="1">
+    <tablePart r:id="rId10"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:H13"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:H18"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="3" customWidth="1"/>
     <col min="2" max="2" width="37" style="3" customWidth="1"/>
@@ -1745,217 +2439,258 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" ht="191.25" customHeight="1"/>
-    <row r="2" spans="1:8">
+    <row r="2" spans="1:8" ht="15">
       <c r="A2" s="4" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="E2" s="4" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="F2" s="4" t="s">
-        <v>25</v>
+        <v>48</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="H2" s="12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" ht="87">
+        <v>49</v>
+      </c>
+      <c r="H2" s="18" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" ht="15">
+      <c r="A3" s="3" t="s">
+        <v>51</v>
+      </c>
+      <c r="B3" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="D3" s="19" t="s">
+        <v>54</v>
+      </c>
+      <c r="E3" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="F3" s="4"/>
+      <c r="G3" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="H3" s="17"/>
+    </row>
+    <row r="4" spans="1:8" s="3" customFormat="1" ht="43.5">
       <c r="A4" s="3" t="s">
-        <v>35</v>
+        <v>57</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>36</v>
+        <v>52</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>37</v>
+        <v>53</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>38</v>
+        <v>58</v>
+      </c>
+      <c r="E4" s="3" t="s">
+        <v>55</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" ht="43.5">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" s="3" customFormat="1" ht="45.75" customHeight="1">
       <c r="A5" s="3" t="s">
-        <v>40</v>
+        <v>60</v>
       </c>
       <c r="B5" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>62</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="E5" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="H5" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="6" spans="1:8" s="3" customFormat="1" ht="16.5" customHeight="1">
+      <c r="A6" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="B6" s="3" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="D6" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="E6" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G6" s="3" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" s="3" customFormat="1" ht="16.5" customHeight="1">
+      <c r="B7" t="s">
+        <v>68</v>
+      </c>
+      <c r="D7" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="E7" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G7" s="3" t="s">
         <v>41</v>
       </c>
-      <c r="C5" s="3" t="s">
-        <v>42</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>39</v>
-      </c>
-      <c r="H5" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8" s="3" customFormat="1" ht="66.75" customHeight="1">
-      <c r="A6" s="3" t="s">
-        <v>45</v>
-      </c>
-      <c r="B6" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="C6" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="D6" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E6" s="3" t="s">
-        <v>49</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" ht="45" customHeight="1">
-      <c r="A7" s="3" t="s">
-        <v>50</v>
-      </c>
-      <c r="B7" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="C7" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="D7" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="E7" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="G7" s="3" t="s">
+    </row>
+    <row r="8" spans="1:8" s="3" customFormat="1" ht="39" customHeight="1">
+      <c r="A8" s="3" t="s">
+        <v>71</v>
+      </c>
+      <c r="B8" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E8" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G8" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="H8" s="3" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" s="3" customFormat="1" ht="39" customHeight="1">
+      <c r="B9" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D9" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="E9" s="3" t="s">
         <v>55</v>
       </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="3" t="s">
+      <c r="G9" s="3" t="s">
+        <v>41</v>
+      </c>
+      <c r="H9" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" s="3" customFormat="1" ht="43.5">
+      <c r="A10" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="B10" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>80</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="E10" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="G10" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H10" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" s="3" customFormat="1" ht="15"/>
+    <row r="12" spans="1:8" s="3" customFormat="1" ht="43.5">
+      <c r="A12" s="3" t="s">
+        <v>83</v>
+      </c>
+      <c r="B12" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>85</v>
+      </c>
+      <c r="D12" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="E12" s="3" t="s">
+        <v>55</v>
+      </c>
+      <c r="G12" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="H12" s="3" t="s">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" s="3" customFormat="1" ht="15"/>
+    <row r="14" spans="1:8" s="3" customFormat="1" ht="29.25">
+      <c r="A14" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="B14" s="3" t="s">
+        <v>88</v>
+      </c>
+      <c r="C14" s="3" t="s">
+        <v>89</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="E14" t="s">
+        <v>91</v>
+      </c>
+      <c r="G14" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="C8" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="G8" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="B9" s="3" t="s">
-        <v>60</v>
-      </c>
-      <c r="C9" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>62</v>
-      </c>
-      <c r="G9" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B10" s="3" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="D10" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="E10" s="3" t="s">
-        <v>67</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="3" t="s">
-        <v>68</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" ht="29.25">
-      <c r="A13" s="3" t="s">
-        <v>63</v>
-      </c>
-      <c r="B13" s="3" t="s">
-        <v>69</v>
-      </c>
-      <c r="C13" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="D13" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G13" s="3" t="s">
-        <v>55</v>
-      </c>
-    </row>
+    </row>
+    <row r="15" spans="1:8" ht="15"/>
+    <row r="16" spans="1:8" ht="15"/>
+    <row r="17" ht="15"/>
+    <row r="18" ht="15"/>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
   <drawing r:id="rId2"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{273AFAA3-99F7-4E93-9580-DCAE2B14D938}">
   <dimension ref="A1:G2"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="19.28515625" customWidth="1"/>
     <col min="2" max="2" width="18.5703125" customWidth="1"/>
@@ -1968,62 +2703,50 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>71</v>
+        <v>92</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>72</v>
+        <v>93</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>21</v>
+        <v>44</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>22</v>
+        <v>45</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>23</v>
+        <v>46</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>24</v>
+        <v>47</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>26</v>
+        <v>49</v>
       </c>
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
-        <v>73</v>
+        <v>94</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>74</v>
+        <v>95</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>75</v>
+        <v>96</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>30</v>
+        <v>97</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>31</v>
+        <v>98</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>32</v>
+        <v>99</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>34</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
-  <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
-  <sheetData>
-    <row r="1" ht="111" customHeight="1"/>
+        <v>100</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
@@ -2031,20 +2754,95 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F2489EBC-5098-4697-9724-F190D24E1C3D}">
+  <dimension ref="A1:D10"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
+  <cols>
+    <col min="1" max="1" width="17.5703125" customWidth="1"/>
+    <col min="2" max="2" width="22" customWidth="1"/>
+    <col min="3" max="3" width="76.5703125" customWidth="1"/>
+    <col min="4" max="4" width="83.28515625" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" ht="111" customHeight="1"/>
+    <row r="2" spans="1:4" ht="15">
+      <c r="A2" s="25" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="26" t="s">
+        <v>102</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="27" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" ht="15">
+      <c r="A3" s="28" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="29" t="s">
+        <v>107</v>
+      </c>
+      <c r="D3" s="30"/>
+    </row>
+    <row r="4" spans="1:4" ht="29.25">
+      <c r="A4" s="28" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="29" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="29" t="s">
+        <v>109</v>
+      </c>
+      <c r="D4" s="30"/>
+    </row>
+    <row r="5" spans="1:4" ht="15">
+      <c r="A5" s="31" t="s">
+        <v>110</v>
+      </c>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31" t="s">
+        <v>111</v>
+      </c>
+      <c r="D5" s="31"/>
+    </row>
+    <row r="6" spans="1:4" ht="15"/>
+    <row r="7" spans="1:4" ht="15"/>
+    <row r="8" spans="1:4" ht="15"/>
+    <row r="9" spans="1:4" ht="15"/>
+    <row r="10" spans="1:4" ht="15"/>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{15D07244-21B1-4120-B673-4A54672CC2AD}">
   <dimension ref="A2:I21"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="2" max="2" width="19.7109375" style="3" customWidth="1"/>
     <col min="3" max="3" width="21.42578125" style="3" customWidth="1"/>
     <col min="4" max="4" width="77.42578125" style="3" customWidth="1"/>
     <col min="5" max="5" width="76.5703125" style="3" customWidth="1"/>
+    <col min="6" max="6" width="44.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="1:9">
       <c r="A2" s="5"/>
       <c r="B2" s="10" t="s">
-        <v>76</v>
+        <v>112</v>
       </c>
       <c r="C2" s="7"/>
       <c r="D2" s="7"/>
@@ -2054,21 +2852,23 @@
       <c r="H2" s="5"/>
       <c r="I2" s="5"/>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" ht="29.25">
       <c r="A3" s="5"/>
       <c r="B3" s="9" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
       <c r="C3" s="9" t="s">
-        <v>78</v>
+        <v>102</v>
       </c>
       <c r="D3" s="9" t="s">
-        <v>79</v>
+        <v>103</v>
       </c>
       <c r="E3" s="11" t="s">
-        <v>80</v>
-      </c>
-      <c r="F3" s="8"/>
+        <v>104</v>
+      </c>
+      <c r="F3" s="20" t="s">
+        <v>50</v>
+      </c>
       <c r="G3" s="8"/>
       <c r="H3" s="8"/>
       <c r="I3" s="5"/>
@@ -2076,134 +2876,216 @@
     <row r="4" spans="1:9" ht="48.75" customHeight="1">
       <c r="A4" s="5"/>
       <c r="B4" s="7" t="s">
-        <v>69</v>
+        <v>88</v>
       </c>
       <c r="C4" s="7" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>82</v>
-      </c>
-      <c r="E4" s="7"/>
-      <c r="F4" s="5"/>
+        <v>114</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>115</v>
+      </c>
+      <c r="F4" s="7"/>
       <c r="G4" s="5"/>
       <c r="H4" s="5"/>
       <c r="I4" s="5"/>
     </row>
-    <row r="5" spans="1:9" ht="29.25">
+    <row r="5" spans="1:9" ht="43.5">
       <c r="B5" s="7" t="s">
-        <v>41</v>
+        <v>116</v>
       </c>
       <c r="C5" s="7" t="s">
-        <v>81</v>
+        <v>113</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>83</v>
-      </c>
-      <c r="E5" s="7"/>
-    </row>
-    <row r="6" spans="1:9">
-      <c r="B6" s="7"/>
+        <v>117</v>
+      </c>
+      <c r="E5" s="7" t="s">
+        <v>118</v>
+      </c>
+      <c r="F5" s="7"/>
+    </row>
+    <row r="6" spans="1:9" ht="29.25">
+      <c r="B6" s="7" t="s">
+        <v>119</v>
+      </c>
       <c r="C6" s="7"/>
       <c r="D6" s="7" t="s">
-        <v>84</v>
-      </c>
-      <c r="E6" s="7"/>
-    </row>
-    <row r="7" spans="1:9">
-      <c r="B7" s="7"/>
-      <c r="C7" s="7"/>
-      <c r="D7" s="7"/>
-      <c r="E7" s="7"/>
-    </row>
-    <row r="8" spans="1:9">
-      <c r="B8" s="7"/>
-      <c r="C8" s="7"/>
-      <c r="D8" s="7"/>
-      <c r="E8" s="7"/>
-    </row>
-    <row r="9" spans="1:9">
-      <c r="B9" s="7"/>
-      <c r="C9" s="7"/>
-      <c r="D9" s="7"/>
-      <c r="E9" s="7"/>
-    </row>
-    <row r="10" spans="1:9">
-      <c r="B10" s="7"/>
-      <c r="C10" s="7"/>
-      <c r="D10" s="7"/>
-      <c r="E10" s="7"/>
-    </row>
-    <row r="11" spans="1:9">
-      <c r="B11" s="7"/>
+        <v>120</v>
+      </c>
+      <c r="E6" s="7" t="s">
+        <v>121</v>
+      </c>
+      <c r="F6" s="7"/>
+    </row>
+    <row r="7" spans="1:9" ht="30.75" customHeight="1">
+      <c r="B7" s="7" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="7" t="s">
+        <v>113</v>
+      </c>
+      <c r="D7" s="7" t="s">
+        <v>123</v>
+      </c>
+      <c r="E7" s="7" t="s">
+        <v>124</v>
+      </c>
+      <c r="F7" s="7"/>
+    </row>
+    <row r="8" spans="1:9" ht="29.25">
+      <c r="B8" s="7" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="7" t="s">
+        <v>126</v>
+      </c>
+      <c r="E8" s="7" t="s">
+        <v>127</v>
+      </c>
+      <c r="F8" s="7" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15">
+      <c r="B9" s="7" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D9" s="7" t="s">
+        <v>107</v>
+      </c>
+      <c r="E9" s="7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F9" s="7"/>
+    </row>
+    <row r="10" spans="1:9" ht="29.25">
+      <c r="B10" s="7" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="7" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="7" t="s">
+        <v>109</v>
+      </c>
+      <c r="E10" s="7" t="s">
+        <v>130</v>
+      </c>
+      <c r="F10" s="7"/>
+    </row>
+    <row r="11" spans="1:9" ht="15">
+      <c r="B11" s="15" t="s">
+        <v>131</v>
+      </c>
       <c r="C11" s="7"/>
-      <c r="D11" s="7"/>
-      <c r="E11" s="7"/>
-    </row>
-    <row r="12" spans="1:9">
-      <c r="B12" s="7"/>
-      <c r="C12" s="7"/>
-      <c r="D12" s="7"/>
+      <c r="D11" s="7" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="7" t="s">
+        <v>133</v>
+      </c>
+      <c r="F11" s="7"/>
+    </row>
+    <row r="12" spans="1:9" ht="29.25">
+      <c r="B12" s="7" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D12" s="7" t="s">
+        <v>136</v>
+      </c>
       <c r="E12" s="7"/>
-    </row>
-    <row r="13" spans="1:9">
-      <c r="B13" s="7"/>
-      <c r="C13" s="7"/>
-      <c r="D13" s="7"/>
+      <c r="F12" s="7" t="s">
+        <v>137</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" ht="15">
+      <c r="B13" s="7" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" t="s">
+        <v>139</v>
+      </c>
       <c r="E13" s="7"/>
-    </row>
-    <row r="14" spans="1:9">
-      <c r="B14" s="7"/>
-      <c r="C14" s="7"/>
-      <c r="D14" s="7"/>
+      <c r="F13" s="7"/>
+    </row>
+    <row r="14" spans="1:9" ht="15">
+      <c r="B14" s="7" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="7" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" t="s">
+        <v>141</v>
+      </c>
       <c r="E14" s="7"/>
-    </row>
-    <row r="15" spans="1:9">
+      <c r="F14" s="7"/>
+    </row>
+    <row r="15" spans="1:9" ht="15">
       <c r="B15" s="7"/>
       <c r="C15" s="7"/>
       <c r="D15" s="7"/>
       <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:9">
+      <c r="F15" s="7"/>
+    </row>
+    <row r="16" spans="1:9" ht="15">
       <c r="B16" s="7"/>
       <c r="C16" s="7"/>
       <c r="D16" s="7"/>
       <c r="E16" s="7"/>
-    </row>
-    <row r="17" spans="2:5">
+      <c r="F16" s="7"/>
+    </row>
+    <row r="17" spans="2:6" ht="15">
       <c r="B17" s="7"/>
       <c r="C17" s="7"/>
       <c r="D17" s="7"/>
       <c r="E17" s="7"/>
-    </row>
-    <row r="18" spans="2:5">
+      <c r="F17" s="7"/>
+    </row>
+    <row r="18" spans="2:6" ht="15">
       <c r="B18" s="7"/>
       <c r="C18" s="7"/>
       <c r="D18" s="7"/>
       <c r="E18" s="7"/>
-    </row>
-    <row r="19" spans="2:5">
+      <c r="F18" s="7"/>
+    </row>
+    <row r="19" spans="2:6" ht="15">
       <c r="B19" s="7"/>
       <c r="C19" s="7"/>
       <c r="D19" s="7"/>
       <c r="E19" s="7"/>
-    </row>
-    <row r="20" spans="2:5">
+      <c r="F19" s="7"/>
+    </row>
+    <row r="20" spans="2:6" ht="15">
       <c r="B20" s="7"/>
       <c r="C20" s="7"/>
       <c r="D20" s="7"/>
       <c r="E20" s="7"/>
-    </row>
-    <row r="21" spans="2:5">
-      <c r="B21" s="7"/>
-      <c r="C21" s="7"/>
-      <c r="D21" s="7"/>
-      <c r="E21" s="7"/>
-    </row>
+      <c r="F20" s="7"/>
+    </row>
+    <row r="21" spans="2:6" ht="15"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B11" r:id="rId1" xr:uid="{D10F429E-6B60-488A-B165-0C4F6F5E7C9B}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId1"/>
+    <tablePart r:id="rId2"/>
   </tableParts>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Organization: removed empty rows and added EU filter row
</commit_message>
<xml_diff>
--- a/input/requirements/Organization.xlsx
+++ b/input/requirements/Organization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Organization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="668" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{EE04BCF3-BF31-4511-8967-42B0CF5ACD00}"/>
+  <xr:revisionPtr revIDLastSave="691" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3198798E-7421-42F7-A0EB-F39B0EB73582}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="553" firstSheet="2" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="553" firstSheet="3" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="185" uniqueCount="142">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="143">
   <si>
     <t>Veld</t>
   </si>
@@ -204,6 +204,9 @@
     <t>Opmerkingen</t>
   </si>
   <si>
+    <t>EU filter</t>
+  </si>
+  <si>
     <t>ORG-001</t>
   </si>
   <si>
@@ -219,7 +222,7 @@
     <t>0..*</t>
   </si>
   <si>
-    <t>Xt-EHR LIM 1.0.0 Organization</t>
+    <t>EHDSOrganization</t>
   </si>
   <si>
     <t>ORG-002</t>
@@ -277,7 +280,7 @@
     <t>(string)</t>
   </si>
   <si>
-    <t>Xt-EHR LIM 1.0.0 Organization, BgZ-MSZ</t>
+    <t>EHDSOrganization, BgZ-MSZ</t>
   </si>
   <si>
     <t xml:space="preserve"> If an identification number is given, the name must match the name that corresponds to the identification number.</t>
@@ -299,7 +302,7 @@
 SHALL An address of an organization can never be of use 'home'</t>
   </si>
   <si>
-    <t>Xt-EHR LIM 1.0.0 Organization, Spoedsamenvatting, BgZ MSZ</t>
+    <t>EHDSOrganization, Spoedsamenvatting, BgZ MSZ</t>
   </si>
   <si>
     <t>ORG-007</t>
@@ -680,14 +683,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -720,15 +720,6 @@
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="1"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -742,31 +733,42 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Standaard" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="29">
+  <dxfs count="30">
     <dxf>
       <font>
         <b val="0"/>
@@ -977,31 +979,35 @@
       <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment wrapText="1"/>
+      <numFmt numFmtId="0" formatCode="General"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1020,7 +1026,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </font>
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <alignment horizontal="left" vertical="top" textRotation="0" wrapText="1" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
       <font>
@@ -1801,21 +1807,21 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{59B5D8CA-526E-41E2-9015-923318959E98}" name="Tabel4" displayName="Tabel4" ref="A2:B11" totalsRowShown="0" headerRowDxfId="28" dataDxfId="27">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="4" xr:uid="{59B5D8CA-526E-41E2-9015-923318959E98}" name="Tabel4" displayName="Tabel4" ref="A2:B11" totalsRowShown="0" headerRowDxfId="29" dataDxfId="28">
   <autoFilter ref="A2:B11" xr:uid="{59B5D8CA-526E-41E2-9015-923318959E98}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{50EFEBF6-4893-432E-BEA1-588A83D972CB}" name="Veld" dataDxfId="26"/>
-    <tableColumn id="2" xr3:uid="{9FB3B455-2F07-4EC4-A31C-65E3885F100A}" name="Beschrijving" dataDxfId="25"/>
+    <tableColumn id="1" xr3:uid="{50EFEBF6-4893-432E-BEA1-588A83D972CB}" name="Veld" dataDxfId="27"/>
+    <tableColumn id="2" xr3:uid="{9FB3B455-2F07-4EC4-A31C-65E3885F100A}" name="Beschrijving" dataDxfId="26"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
 <file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AE4E70E2-B46F-4B62-81CF-884CAD44739D}" name="Tabel5" displayName="Tabel5" ref="A1:C11" totalsRowShown="0" headerRowDxfId="24">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{AE4E70E2-B46F-4B62-81CF-884CAD44739D}" name="Tabel5" displayName="Tabel5" ref="A1:C11" totalsRowShown="0" headerRowDxfId="25">
   <autoFilter ref="A1:C11" xr:uid="{AE4E70E2-B46F-4B62-81CF-884CAD44739D}"/>
   <tableColumns count="3">
-    <tableColumn id="1" xr3:uid="{353B1C84-B074-472C-8FDA-BF6BED2D63C8}" name="type bron" dataDxfId="23"/>
+    <tableColumn id="1" xr3:uid="{353B1C84-B074-472C-8FDA-BF6BED2D63C8}" name="type bron" dataDxfId="24"/>
     <tableColumn id="2" xr3:uid="{0B17EAA3-957B-45FC-A6C7-6D847A216C50}" name="link" dataCellStyle="Hyperlink"/>
     <tableColumn id="3" xr3:uid="{8B33B7A8-D1F0-4831-95B4-64521C7111E4}" name="aantekeningen"/>
   </tableColumns>
@@ -1824,17 +1830,20 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}" name="Tabel2" displayName="Tabel2" ref="A2:H14" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
-  <autoFilter ref="A2:H14" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}"/>
-  <tableColumns count="8">
-    <tableColumn id="1" xr3:uid="{AEDCF761-C41E-45F9-8585-F195D983B89C}" name="Nummer" dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{635CD206-F27E-4A6A-BC65-EEED36933D1E}" name="Naam" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{8EF3A9D6-055E-4CB8-96A3-6552DF1766C8}" name="Omschrijving" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{C3044835-AC84-438A-ADC2-CAD99CE92BD0}" name="Variabiliteit" dataDxfId="17"/>
-    <tableColumn id="5" xr3:uid="{AA18877F-FB5A-4805-A5CF-69206661B387}" name="Aanwezigheid" dataDxfId="16"/>
-    <tableColumn id="6" xr3:uid="{564C5C8F-5623-4C63-8144-810E58143EDA}" name="Verleden/heden/toekomst" dataDxfId="15"/>
-    <tableColumn id="7" xr3:uid="{58DBAFD8-EA1C-440F-9872-7271A13F1C90}" name="Herkomst" dataDxfId="14"/>
-    <tableColumn id="8" xr3:uid="{F805880C-4939-45E5-9047-13B213C612A8}" name="Opmerkingen" dataDxfId="13"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}" name="Tabel2" displayName="Tabel2" ref="A2:I12" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="A2:I12" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}"/>
+  <tableColumns count="9">
+    <tableColumn id="1" xr3:uid="{AEDCF761-C41E-45F9-8585-F195D983B89C}" name="Nummer" dataDxfId="21"/>
+    <tableColumn id="2" xr3:uid="{635CD206-F27E-4A6A-BC65-EEED36933D1E}" name="Naam" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{8EF3A9D6-055E-4CB8-96A3-6552DF1766C8}" name="Omschrijving" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{C3044835-AC84-438A-ADC2-CAD99CE92BD0}" name="Variabiliteit" dataDxfId="18"/>
+    <tableColumn id="5" xr3:uid="{AA18877F-FB5A-4805-A5CF-69206661B387}" name="Aanwezigheid" dataDxfId="17"/>
+    <tableColumn id="6" xr3:uid="{564C5C8F-5623-4C63-8144-810E58143EDA}" name="Verleden/heden/toekomst" dataDxfId="16"/>
+    <tableColumn id="7" xr3:uid="{58DBAFD8-EA1C-440F-9872-7271A13F1C90}" name="Herkomst" dataDxfId="15"/>
+    <tableColumn id="8" xr3:uid="{F805880C-4939-45E5-9047-13B213C612A8}" name="Opmerkingen" dataDxfId="14"/>
+    <tableColumn id="9" xr3:uid="{B16F7E82-08F9-401A-8EA3-02C7E15C7DC3}" name="EU filter" dataDxfId="13">
+      <calculatedColumnFormula>ISNUMBER(SEARCH("EHDS", G3))</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium3" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -2212,82 +2221,82 @@
       <c r="A1" s="3"/>
     </row>
     <row r="2" spans="1:2" ht="15">
-      <c r="A2" s="21" t="s">
+      <c r="A2" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="21" t="s">
+      <c r="B2" s="17" t="s">
         <v>1</v>
       </c>
     </row>
     <row r="3" spans="1:2" ht="15">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="18" t="s">
         <v>2</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="18" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="4" spans="1:2" ht="43.5">
-      <c r="A4" s="22" t="s">
+      <c r="A4" s="18" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="22" t="s">
+      <c r="B4" s="18" t="s">
         <v>5</v>
       </c>
     </row>
     <row r="5" spans="1:2" ht="15">
-      <c r="A5" s="22" t="s">
+      <c r="A5" s="18" t="s">
         <v>6</v>
       </c>
-      <c r="B5" s="22" t="s">
+      <c r="B5" s="18" t="s">
         <v>7</v>
       </c>
     </row>
     <row r="6" spans="1:2" ht="15">
-      <c r="A6" s="22" t="s">
+      <c r="A6" s="18" t="s">
         <v>8</v>
       </c>
-      <c r="B6" s="22" t="s">
+      <c r="B6" s="18" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="7" spans="1:2" ht="15">
-      <c r="A7" s="22" t="s">
+      <c r="A7" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="B7" s="22" t="s">
+      <c r="B7" s="18" t="s">
         <v>11</v>
       </c>
     </row>
     <row r="8" spans="1:2" ht="138.75" customHeight="1">
-      <c r="A8" s="22" t="s">
+      <c r="A8" s="18" t="s">
         <v>12</v>
       </c>
-      <c r="B8" s="22" t="s">
+      <c r="B8" s="18" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="9" spans="1:2" ht="15">
-      <c r="A9" s="22" t="s">
+      <c r="A9" s="18" t="s">
         <v>14</v>
       </c>
-      <c r="B9" s="22" t="s">
+      <c r="B9" s="18" t="s">
         <v>15</v>
       </c>
     </row>
     <row r="10" spans="1:2" ht="15">
-      <c r="A10" s="22" t="s">
+      <c r="A10" s="18" t="s">
         <v>16</v>
       </c>
-      <c r="B10" s="22" t="s">
+      <c r="B10" s="18" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="11" spans="1:2" ht="15">
-      <c r="A11" s="22" t="s">
+      <c r="A11" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="B11" s="23" t="s">
+      <c r="B11" s="19" t="s">
         <v>19</v>
       </c>
     </row>
@@ -2311,95 +2320,95 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:3">
-      <c r="A1" s="12" t="s">
+      <c r="A1" s="11" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="12" t="s">
+      <c r="B1" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="C1" s="12" t="s">
+      <c r="C1" s="11" t="s">
         <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:3" ht="15">
-      <c r="A2" s="13" t="s">
+      <c r="A2" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="B2" s="14" t="s">
+      <c r="B2" s="13" t="s">
         <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:3" ht="29.25">
-      <c r="A3" s="13" t="s">
+      <c r="A3" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="13" t="s">
         <v>26</v>
       </c>
     </row>
     <row r="4" spans="1:3" ht="15">
-      <c r="A4" s="13" t="s">
+      <c r="A4" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="14" t="s">
         <v>28</v>
       </c>
-      <c r="C4" s="24" t="s">
+      <c r="C4" s="20" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:3" ht="29.25">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="B5" s="14" t="s">
+      <c r="B5" s="13" t="s">
         <v>31</v>
       </c>
-      <c r="C5" s="16"/>
+      <c r="C5" s="15"/>
     </row>
     <row r="6" spans="1:3" ht="29.25">
-      <c r="A6" s="13" t="s">
+      <c r="A6" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="14" t="s">
+      <c r="B6" s="13" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7" spans="1:3" ht="28.9">
-      <c r="A7" s="13" t="s">
+      <c r="A7" s="12" t="s">
         <v>34</v>
       </c>
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="14" t="s">
         <v>35</v>
       </c>
     </row>
     <row r="8" spans="1:3" ht="28.9">
-      <c r="A8" s="13" t="s">
+      <c r="A8" s="12" t="s">
         <v>36</v>
       </c>
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="14" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="9" spans="1:3" ht="43.15">
-      <c r="A9" s="13" t="s">
+      <c r="A9" s="12" t="s">
         <v>38</v>
       </c>
-      <c r="B9" s="15" t="s">
+      <c r="B9" s="14" t="s">
         <v>39</v>
       </c>
     </row>
     <row r="10" spans="1:3" ht="28.9">
-      <c r="A10" s="13" t="s">
+      <c r="A10" s="12" t="s">
         <v>40</v>
       </c>
-      <c r="B10" s="14"/>
+      <c r="B10" s="13"/>
     </row>
     <row r="11" spans="1:3" ht="15">
       <c r="A11" t="s">
         <v>41</v>
       </c>
-      <c r="B11" s="15" t="s">
+      <c r="B11" s="14" t="s">
         <v>42</v>
       </c>
     </row>
@@ -2425,257 +2434,296 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:H18"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <dimension ref="A1:I12"/>
+  <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="13.28515625" style="3" customWidth="1"/>
-    <col min="2" max="2" width="37" style="3" customWidth="1"/>
-    <col min="3" max="3" width="68.42578125" style="3" customWidth="1"/>
-    <col min="4" max="4" width="52.140625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="54" style="3" customWidth="1"/>
-    <col min="6" max="6" width="48.7109375" style="3" customWidth="1"/>
-    <col min="7" max="7" width="34.42578125" style="3" customWidth="1"/>
-    <col min="8" max="8" width="39.5703125" customWidth="1"/>
+    <col min="1" max="1" width="13.28515625" style="18" customWidth="1"/>
+    <col min="2" max="2" width="37" style="18" customWidth="1"/>
+    <col min="3" max="3" width="68.42578125" style="18" customWidth="1"/>
+    <col min="4" max="4" width="52.140625" style="18" customWidth="1"/>
+    <col min="5" max="5" width="54" style="18" customWidth="1"/>
+    <col min="6" max="6" width="48.7109375" style="18" customWidth="1"/>
+    <col min="7" max="7" width="34.42578125" style="18" customWidth="1"/>
+    <col min="8" max="8" width="39.5703125" style="18" customWidth="1"/>
+    <col min="9" max="9" width="39.7109375" style="18" customWidth="1"/>
+    <col min="10" max="16384" width="9.140625" style="18"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="191.25" customHeight="1"/>
-    <row r="2" spans="1:8" ht="15">
-      <c r="A2" s="4" t="s">
+    <row r="1" spans="1:9" ht="191.25" customHeight="1"/>
+    <row r="2" spans="1:9">
+      <c r="A2" s="17" t="s">
         <v>43</v>
       </c>
-      <c r="B2" s="4" t="s">
+      <c r="B2" s="17" t="s">
         <v>44</v>
       </c>
-      <c r="C2" s="4" t="s">
+      <c r="C2" s="17" t="s">
         <v>45</v>
       </c>
-      <c r="D2" s="4" t="s">
+      <c r="D2" s="17" t="s">
         <v>46</v>
       </c>
-      <c r="E2" s="4" t="s">
+      <c r="E2" s="17" t="s">
         <v>47</v>
       </c>
-      <c r="F2" s="4" t="s">
+      <c r="F2" s="17" t="s">
         <v>48</v>
       </c>
-      <c r="G2" s="4" t="s">
+      <c r="G2" s="17" t="s">
         <v>49</v>
       </c>
-      <c r="H2" s="18" t="s">
+      <c r="H2" s="27" t="s">
         <v>50</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" ht="15">
-      <c r="A3" s="3" t="s">
+      <c r="I2" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="B3" s="3" t="s">
+    </row>
+    <row r="3" spans="1:9">
+      <c r="A3" s="18" t="s">
         <v>52</v>
       </c>
-      <c r="C3" s="3" t="s">
+      <c r="B3" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="C3" s="18" t="s">
         <v>54</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="D3" s="6" t="s">
         <v>55</v>
       </c>
-      <c r="F3" s="4"/>
-      <c r="G3" s="3" t="s">
+      <c r="E3" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="H3" s="17"/>
-    </row>
-    <row r="4" spans="1:8" s="3" customFormat="1" ht="43.5">
-      <c r="A4" s="3" t="s">
+      <c r="F3" s="17"/>
+      <c r="G3" s="18" t="s">
         <v>57</v>
       </c>
-      <c r="B4" s="3" t="s">
-        <v>52</v>
-      </c>
-      <c r="C4" s="3" t="s">
+      <c r="H3" s="28"/>
+      <c r="I3" s="29" t="b">
+        <f t="shared" ref="I3:I12" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="43.5">
+      <c r="A4" s="18" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="18" t="s">
         <v>53</v>
       </c>
-      <c r="D4" s="3" t="s">
-        <v>58</v>
-      </c>
-      <c r="E4" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G4" s="3" t="s">
+      <c r="C4" s="18" t="s">
+        <v>54</v>
+      </c>
+      <c r="D4" s="18" t="s">
         <v>59</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" s="3" customFormat="1" ht="45.75" customHeight="1">
-      <c r="A5" s="3" t="s">
+      <c r="E4" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G4" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="3" t="s">
+      <c r="I4" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="45.75" customHeight="1">
+      <c r="A5" s="18" t="s">
         <v>61</v>
       </c>
-      <c r="C5" s="3" t="s">
+      <c r="B5" s="18" t="s">
         <v>62</v>
       </c>
-      <c r="D5" s="3" t="s">
+      <c r="C5" s="18" t="s">
         <v>63</v>
       </c>
-      <c r="E5" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G5" s="3" t="s">
-        <v>59</v>
-      </c>
-      <c r="H5" t="s">
+      <c r="D5" s="18" t="s">
         <v>64</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" s="3" customFormat="1" ht="16.5" customHeight="1">
-      <c r="A6" s="3" t="s">
+      <c r="E5" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G5" s="18" t="s">
+        <v>60</v>
+      </c>
+      <c r="H5" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="B6" s="3" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="3" t="s">
+      <c r="I5" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="16.5" customHeight="1">
+      <c r="A6" s="18" t="s">
         <v>66</v>
       </c>
-      <c r="D6" s="3" t="s">
+      <c r="B6" s="18" t="s">
+        <v>62</v>
+      </c>
+      <c r="C6" s="18" t="s">
         <v>67</v>
       </c>
-      <c r="E6" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G6" s="3" t="s">
+      <c r="D6" s="18" t="s">
+        <v>68</v>
+      </c>
+      <c r="E6" s="18" t="s">
         <v>56</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" s="3" customFormat="1" ht="16.5" customHeight="1">
-      <c r="B7" t="s">
-        <v>68</v>
-      </c>
-      <c r="D7" s="3" t="s">
+      <c r="G6" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="I6" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="16.5" customHeight="1">
+      <c r="B7" s="18" t="s">
         <v>69</v>
       </c>
-      <c r="E7" s="3" t="s">
+      <c r="D7" s="18" t="s">
         <v>70</v>
       </c>
-      <c r="G7" s="3" t="s">
+      <c r="E7" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G7" s="18" t="s">
         <v>41</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" s="3" customFormat="1" ht="39" customHeight="1">
-      <c r="A8" s="3" t="s">
+      <c r="I7" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="39" customHeight="1">
+      <c r="A8" s="18" t="s">
+        <v>72</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>74</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>75</v>
+      </c>
+      <c r="E8" s="18" t="s">
         <v>71</v>
       </c>
-      <c r="B8" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="C8" s="3" t="s">
+      <c r="G8" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="I8" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="39" customHeight="1">
+      <c r="B9" s="18" t="s">
         <v>73</v>
       </c>
-      <c r="D8" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E8" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G8" s="3" t="s">
+      <c r="D9" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="H8" s="3" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" s="3" customFormat="1" ht="39" customHeight="1">
-      <c r="B9" s="3" t="s">
-        <v>72</v>
-      </c>
-      <c r="D9" s="3" t="s">
-        <v>74</v>
-      </c>
-      <c r="E9" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G9" s="3" t="s">
+      <c r="E9" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G9" s="18" t="s">
         <v>41</v>
       </c>
-      <c r="H9" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" s="3" customFormat="1" ht="43.5">
-      <c r="A10" s="3" t="s">
+      <c r="H9" s="18" t="s">
         <v>78</v>
       </c>
-      <c r="B10" s="3" t="s">
+      <c r="I9" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="43.5">
+      <c r="A10" s="18" t="s">
         <v>79</v>
       </c>
-      <c r="C10" s="3" t="s">
+      <c r="B10" s="18" t="s">
         <v>80</v>
       </c>
-      <c r="D10" s="3" t="s">
+      <c r="C10" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="E10" s="3" t="s">
-        <v>70</v>
-      </c>
-      <c r="G10" s="3" t="s">
+      <c r="D10" s="18" t="s">
         <v>82</v>
       </c>
-      <c r="H10" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" s="3" customFormat="1" ht="15"/>
-    <row r="12" spans="1:8" s="3" customFormat="1" ht="43.5">
-      <c r="A12" s="3" t="s">
+      <c r="E10" s="18" t="s">
+        <v>71</v>
+      </c>
+      <c r="G10" s="18" t="s">
         <v>83</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="H10" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="I10" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="43.5">
+      <c r="A11" s="18" t="s">
         <v>84</v>
       </c>
-      <c r="C12" s="3" t="s">
+      <c r="B11" s="18" t="s">
         <v>85</v>
       </c>
-      <c r="D12" s="3" t="s">
+      <c r="C11" s="18" t="s">
         <v>86</v>
       </c>
-      <c r="E12" s="3" t="s">
-        <v>55</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>82</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>77</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" s="3" customFormat="1" ht="15"/>
-    <row r="14" spans="1:8" s="3" customFormat="1" ht="29.25">
-      <c r="A14" s="3" t="s">
+      <c r="D11" s="18" t="s">
         <v>87</v>
       </c>
-      <c r="B14" s="3" t="s">
+      <c r="E11" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="G11" s="18" t="s">
+        <v>83</v>
+      </c>
+      <c r="H11" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="I11" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" ht="43.5">
+      <c r="A12" s="18" t="s">
         <v>88</v>
       </c>
-      <c r="C14" s="3" t="s">
+      <c r="B12" s="18" t="s">
         <v>89</v>
       </c>
-      <c r="D14" s="3" t="s">
+      <c r="C12" s="18" t="s">
         <v>90</v>
       </c>
-      <c r="E14" t="s">
+      <c r="D12" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="G14" s="3" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8" ht="15"/>
-    <row r="16" spans="1:8" ht="15"/>
-    <row r="17" ht="15"/>
-    <row r="18" ht="15"/>
+      <c r="E12" s="18" t="s">
+        <v>92</v>
+      </c>
+      <c r="G12" s="30" t="s">
+        <v>57</v>
+      </c>
+      <c r="I12" s="29" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
   </sheetData>
   <phoneticPr fontId="3" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -2703,10 +2751,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1">
       <c r="A1" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>44</v>
@@ -2726,25 +2774,25 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2766,52 +2814,50 @@
   <sheetData>
     <row r="1" spans="1:4" ht="111" customHeight="1"/>
     <row r="2" spans="1:4" ht="15">
-      <c r="A2" s="25" t="s">
-        <v>101</v>
-      </c>
-      <c r="B2" s="26" t="s">
+      <c r="A2" s="21" t="s">
         <v>102</v>
       </c>
-      <c r="C2" s="26" t="s">
+      <c r="B2" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="C2" s="22" t="s">
         <v>104</v>
       </c>
+      <c r="D2" s="23" t="s">
+        <v>105</v>
+      </c>
     </row>
     <row r="3" spans="1:4" ht="15">
-      <c r="A3" s="28" t="s">
-        <v>105</v>
-      </c>
-      <c r="B3" s="29" t="s">
+      <c r="A3" s="24" t="s">
         <v>106</v>
       </c>
-      <c r="C3" s="29" t="s">
+      <c r="B3" s="25" t="s">
         <v>107</v>
       </c>
-      <c r="D3" s="30"/>
+      <c r="C3" s="25" t="s">
+        <v>108</v>
+      </c>
+      <c r="D3" s="26"/>
     </row>
     <row r="4" spans="1:4" ht="29.25">
-      <c r="A4" s="28" t="s">
-        <v>108</v>
-      </c>
-      <c r="B4" s="29" t="s">
-        <v>106</v>
-      </c>
-      <c r="C4" s="29" t="s">
+      <c r="A4" s="24" t="s">
         <v>109</v>
       </c>
-      <c r="D4" s="30"/>
+      <c r="B4" s="25" t="s">
+        <v>107</v>
+      </c>
+      <c r="C4" s="25" t="s">
+        <v>110</v>
+      </c>
+      <c r="D4" s="26"/>
     </row>
     <row r="5" spans="1:4" ht="15">
-      <c r="A5" s="31" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="31"/>
-      <c r="C5" s="31" t="s">
+      <c r="A5" t="s">
         <v>111</v>
       </c>
-      <c r="D5" s="31"/>
+      <c r="C5" t="s">
+        <v>112</v>
+      </c>
     </row>
     <row r="6" spans="1:4" ht="15"/>
     <row r="7" spans="1:4" ht="15"/>
@@ -2840,243 +2886,243 @@
   </cols>
   <sheetData>
     <row r="2" spans="1:9">
-      <c r="A2" s="5"/>
-      <c r="B2" s="10" t="s">
-        <v>112</v>
-      </c>
-      <c r="C2" s="7"/>
-      <c r="D2" s="7"/>
-      <c r="E2" s="7"/>
-      <c r="F2" s="6"/>
-      <c r="G2" s="5"/>
-      <c r="H2" s="5"/>
-      <c r="I2" s="5"/>
+      <c r="A2" s="4"/>
+      <c r="B2" s="9" t="s">
+        <v>113</v>
+      </c>
+      <c r="C2" s="6"/>
+      <c r="D2" s="6"/>
+      <c r="E2" s="6"/>
+      <c r="F2" s="5"/>
+      <c r="G2" s="4"/>
+      <c r="H2" s="4"/>
+      <c r="I2" s="4"/>
     </row>
     <row r="3" spans="1:9" ht="29.25">
-      <c r="A3" s="5"/>
-      <c r="B3" s="9" t="s">
-        <v>101</v>
-      </c>
-      <c r="C3" s="9" t="s">
+      <c r="A3" s="4"/>
+      <c r="B3" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="D3" s="9" t="s">
+      <c r="C3" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="E3" s="11" t="s">
+      <c r="D3" s="8" t="s">
         <v>104</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="E3" s="10" t="s">
+        <v>105</v>
+      </c>
+      <c r="F3" s="16" t="s">
         <v>50</v>
       </c>
-      <c r="G3" s="8"/>
-      <c r="H3" s="8"/>
-      <c r="I3" s="5"/>
+      <c r="G3" s="7"/>
+      <c r="H3" s="7"/>
+      <c r="I3" s="4"/>
     </row>
     <row r="4" spans="1:9" ht="48.75" customHeight="1">
-      <c r="A4" s="5"/>
-      <c r="B4" s="7" t="s">
-        <v>88</v>
-      </c>
-      <c r="C4" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="D4" s="7" t="s">
+      <c r="A4" s="4"/>
+      <c r="B4" s="6" t="s">
+        <v>89</v>
+      </c>
+      <c r="C4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="E4" s="7" t="s">
+      <c r="D4" s="6" t="s">
         <v>115</v>
       </c>
-      <c r="F4" s="7"/>
-      <c r="G4" s="5"/>
-      <c r="H4" s="5"/>
-      <c r="I4" s="5"/>
+      <c r="E4" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="F4" s="6"/>
+      <c r="G4" s="4"/>
+      <c r="H4" s="4"/>
+      <c r="I4" s="4"/>
     </row>
     <row r="5" spans="1:9" ht="43.5">
-      <c r="B5" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="C5" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="D5" s="7" t="s">
+      <c r="B5" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="E5" s="7" t="s">
+      <c r="C5" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>118</v>
       </c>
-      <c r="F5" s="7"/>
+      <c r="E5" s="6" t="s">
+        <v>119</v>
+      </c>
+      <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:9" ht="29.25">
-      <c r="B6" s="7" t="s">
-        <v>119</v>
-      </c>
-      <c r="C6" s="7"/>
-      <c r="D6" s="7" t="s">
+      <c r="B6" s="6" t="s">
         <v>120</v>
       </c>
-      <c r="E6" s="7" t="s">
+      <c r="C6" s="6"/>
+      <c r="D6" s="6" t="s">
         <v>121</v>
       </c>
-      <c r="F6" s="7"/>
+      <c r="E6" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:9" ht="30.75" customHeight="1">
-      <c r="B7" s="7" t="s">
-        <v>122</v>
-      </c>
-      <c r="C7" s="7" t="s">
-        <v>113</v>
-      </c>
-      <c r="D7" s="7" t="s">
+      <c r="B7" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="E7" s="7" t="s">
+      <c r="C7" s="6" t="s">
+        <v>114</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>124</v>
       </c>
-      <c r="F7" s="7"/>
+      <c r="E7" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:9" ht="29.25">
-      <c r="B8" s="7" t="s">
-        <v>125</v>
-      </c>
-      <c r="C8" s="7" t="s">
+      <c r="B8" s="6" t="s">
+        <v>126</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D8" s="6" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="6" t="s">
+        <v>128</v>
+      </c>
+      <c r="F8" s="6" t="s">
+        <v>129</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15">
+      <c r="B9" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="D8" s="7" t="s">
-        <v>126</v>
-      </c>
-      <c r="E8" s="7" t="s">
-        <v>127</v>
-      </c>
-      <c r="F8" s="7" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="9" spans="1:9" ht="15">
-      <c r="B9" s="7" t="s">
-        <v>105</v>
-      </c>
-      <c r="C9" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D9" s="7" t="s">
+      <c r="C9" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="E9" s="7" t="s">
-        <v>129</v>
-      </c>
-      <c r="F9" s="7"/>
+      <c r="D9" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="E9" s="6" t="s">
+        <v>130</v>
+      </c>
+      <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:9" ht="29.25">
-      <c r="B10" s="7" t="s">
-        <v>108</v>
-      </c>
-      <c r="C10" s="7" t="s">
-        <v>106</v>
-      </c>
-      <c r="D10" s="7" t="s">
+      <c r="B10" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="E10" s="7" t="s">
-        <v>130</v>
-      </c>
-      <c r="F10" s="7"/>
+      <c r="C10" s="6" t="s">
+        <v>107</v>
+      </c>
+      <c r="D10" s="6" t="s">
+        <v>110</v>
+      </c>
+      <c r="E10" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:9" ht="15">
-      <c r="B11" s="15" t="s">
-        <v>131</v>
-      </c>
-      <c r="C11" s="7"/>
-      <c r="D11" s="7" t="s">
+      <c r="B11" s="14" t="s">
         <v>132</v>
       </c>
-      <c r="E11" s="7" t="s">
+      <c r="C11" s="6"/>
+      <c r="D11" s="6" t="s">
         <v>133</v>
       </c>
-      <c r="F11" s="7"/>
+      <c r="E11" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="29.25">
-      <c r="B12" s="7" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="7" t="s">
+      <c r="B12" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="D12" s="7" t="s">
+      <c r="C12" s="6" t="s">
         <v>136</v>
       </c>
-      <c r="E12" s="7"/>
-      <c r="F12" s="7" t="s">
+      <c r="D12" s="6" t="s">
         <v>137</v>
       </c>
+      <c r="E12" s="6"/>
+      <c r="F12" s="6" t="s">
+        <v>138</v>
+      </c>
     </row>
     <row r="13" spans="1:9" ht="15">
-      <c r="B13" s="7" t="s">
-        <v>138</v>
-      </c>
-      <c r="C13" s="7" t="s">
-        <v>135</v>
+      <c r="B13" s="6" t="s">
+        <v>139</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>136</v>
       </c>
       <c r="D13" t="s">
-        <v>139</v>
-      </c>
-      <c r="E13" s="7"/>
-      <c r="F13" s="7"/>
+        <v>140</v>
+      </c>
+      <c r="E13" s="6"/>
+      <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:9" ht="15">
-      <c r="B14" s="7" t="s">
-        <v>140</v>
-      </c>
-      <c r="C14" s="7" t="s">
-        <v>135</v>
+      <c r="B14" s="6" t="s">
+        <v>141</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>136</v>
       </c>
       <c r="D14" t="s">
-        <v>141</v>
-      </c>
-      <c r="E14" s="7"/>
-      <c r="F14" s="7"/>
+        <v>142</v>
+      </c>
+      <c r="E14" s="6"/>
+      <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:9" ht="15">
-      <c r="B15" s="7"/>
-      <c r="C15" s="7"/>
-      <c r="D15" s="7"/>
-      <c r="E15" s="7"/>
-      <c r="F15" s="7"/>
+      <c r="B15" s="6"/>
+      <c r="C15" s="6"/>
+      <c r="D15" s="6"/>
+      <c r="E15" s="6"/>
+      <c r="F15" s="6"/>
     </row>
     <row r="16" spans="1:9" ht="15">
-      <c r="B16" s="7"/>
-      <c r="C16" s="7"/>
-      <c r="D16" s="7"/>
-      <c r="E16" s="7"/>
-      <c r="F16" s="7"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
+      <c r="F16" s="6"/>
     </row>
     <row r="17" spans="2:6" ht="15">
-      <c r="B17" s="7"/>
-      <c r="C17" s="7"/>
-      <c r="D17" s="7"/>
-      <c r="E17" s="7"/>
-      <c r="F17" s="7"/>
+      <c r="B17" s="6"/>
+      <c r="C17" s="6"/>
+      <c r="D17" s="6"/>
+      <c r="E17" s="6"/>
+      <c r="F17" s="6"/>
     </row>
     <row r="18" spans="2:6" ht="15">
-      <c r="B18" s="7"/>
-      <c r="C18" s="7"/>
-      <c r="D18" s="7"/>
-      <c r="E18" s="7"/>
-      <c r="F18" s="7"/>
+      <c r="B18" s="6"/>
+      <c r="C18" s="6"/>
+      <c r="D18" s="6"/>
+      <c r="E18" s="6"/>
+      <c r="F18" s="6"/>
     </row>
     <row r="19" spans="2:6" ht="15">
-      <c r="B19" s="7"/>
-      <c r="C19" s="7"/>
-      <c r="D19" s="7"/>
-      <c r="E19" s="7"/>
-      <c r="F19" s="7"/>
+      <c r="B19" s="6"/>
+      <c r="C19" s="6"/>
+      <c r="D19" s="6"/>
+      <c r="E19" s="6"/>
+      <c r="F19" s="6"/>
     </row>
     <row r="20" spans="2:6" ht="15">
-      <c r="B20" s="7"/>
-      <c r="C20" s="7"/>
-      <c r="D20" s="7"/>
-      <c r="E20" s="7"/>
-      <c r="F20" s="7"/>
+      <c r="B20" s="6"/>
+      <c r="C20" s="6"/>
+      <c r="D20" s="6"/>
+      <c r="E20" s="6"/>
+      <c r="F20" s="6"/>
     </row>
     <row r="21" spans="2:6" ht="15"/>
   </sheetData>
@@ -3091,15 +3137,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3306,6 +3343,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3318,11 +3364,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>

<commit_message>
Organization: fixed nullpointer error by removing rows with empty requirement id
</commit_message>
<xml_diff>
--- a/input/requirements/Organization.xlsx
+++ b/input/requirements/Organization.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://nictiznl.sharepoint.com/sites/Zib-transitiecommunity/Gedeelde documenten/Architectuur/Werkgroepen ZIBS 2.0 Implementatie/Bouwblokken/Organization/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="691" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3198798E-7421-42F7-A0EB-F39B0EB73582}"/>
+  <xr:revisionPtr revIDLastSave="714" documentId="8_{14C11024-DAA1-4BC8-A0C0-1702803526E6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C1ABF9D3-352C-42C2-B6E8-5C0A7CA1CFEE}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="553" firstSheet="3" activeTab="3" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="553" firstSheet="3" activeTab="6" xr2:uid="{71855D19-E937-4D4D-85D2-5BCEBB780255}"/>
   </bookViews>
   <sheets>
     <sheet name="Uitleg" sheetId="5" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="186" uniqueCount="143">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="182" uniqueCount="146">
   <si>
     <t>Veld</t>
   </si>
@@ -232,7 +232,7 @@
 SHOULD For Dutch healthcare providers, the URA number or the AGB number is used, if possible.</t>
   </si>
   <si>
-    <t>Zib2020, Spoedsamenvatting, BgZ-MSZ</t>
+    <t>Zib2020, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
   </si>
   <si>
     <t>ORG-003</t>
@@ -259,34 +259,25 @@
     <t>Binding Description: (preferred): HL7 organisation_type</t>
   </si>
   <si>
-    <t>hl7:standardIndustryClassCode</t>
-  </si>
-  <si>
-    <t>OrganizationIndustryClass</t>
+    <t>ORG-005</t>
+  </si>
+  <si>
+    <t>OrganizationName</t>
+  </si>
+  <si>
+    <t>Name of the organization.</t>
+  </si>
+  <si>
+    <t>(string)</t>
   </si>
   <si>
     <t>0..1</t>
   </si>
   <si>
-    <t>ORG-005</t>
-  </si>
-  <si>
-    <t>OrganizationName</t>
-  </si>
-  <si>
-    <t>Name of the organization.</t>
-  </si>
-  <si>
-    <t>(string)</t>
-  </si>
-  <si>
-    <t>EHDSOrganization, BgZ-MSZ</t>
+    <t>EHDSOrganization, BgZ-MSZ 2.0</t>
   </si>
   <si>
     <t xml:space="preserve"> If an identification number is given, the name must match the name that corresponds to the identification number.</t>
-  </si>
-  <si>
-    <t>Zie discussie</t>
   </si>
   <si>
     <t>ORG-006</t>
@@ -302,7 +293,10 @@
 SHALL An address of an organization can never be of use 'home'</t>
   </si>
   <si>
-    <t>EHDSOrganization, Spoedsamenvatting, BgZ MSZ</t>
+    <t>EHDSOrganization, Spoedsamenvatting 2.2.0, BgZ MSZ 2.0</t>
+  </si>
+  <si>
+    <t>Zie discussie</t>
   </si>
   <si>
     <t>ORG-007</t>
@@ -318,6 +312,9 @@
 SHALL The telecom of an organization can never be of use 'home'</t>
   </si>
   <si>
+    <t>EHDSOrganization, Spoedsamenvatting 2.2.0, BgZ-MSZ 2.0</t>
+  </si>
+  <si>
     <t>ORG-008</t>
   </si>
   <si>
@@ -465,7 +462,7 @@
     <t>SSV</t>
   </si>
   <si>
-    <t>In de SSV meerdere namen mogelijk, kardinaliteit 0..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat (in het FHIR profiel is .name 1..1)</t>
+    <t>In de SSV meerdere namen mogelijk, kardinaliteit 1..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat (in het FHIR profiel is .name 1..1)</t>
   </si>
   <si>
     <t>Organization.name aankaarten bij FHIR EU, omdat deze 1..1 ipv de LIM die aangeeft dat deze 0..1 is.</t>
@@ -481,6 +478,18 @@
   </si>
   <si>
     <t>In de SSV meerdere Telecom mogelijk, kardinaliteit 0..*, terwijl EHDS LIM (en GBB afsprakenmodel) op 0..1 staat. Dit wordt opgelost als de modeleering vanuit R% teruggezet wordt naar R4 (zonder contact container)</t>
+  </si>
+  <si>
+    <t>EU base</t>
+  </si>
+  <si>
+    <t>Kardinaliteit verschil tussen LIM en FHIR profiel LIM = 1..1 Profile = 0..1</t>
+  </si>
+  <si>
+    <t>Ticket aangemaakt op HL7 jira omgeving</t>
+  </si>
+  <si>
+    <t>Link: https://jira.hl7.org/browse/FHIR-58618</t>
   </si>
 </sst>
 </file>
@@ -683,7 +692,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="31">
+  <cellXfs count="30">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -755,9 +764,6 @@
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -1830,8 +1836,8 @@
 </file>
 
 <file path=xl/tables/table3.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}" name="Tabel2" displayName="Tabel2" ref="A2:I12" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
-  <autoFilter ref="A2:I12" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="2" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}" name="Tabel2" displayName="Tabel2" ref="A2:I10" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+  <autoFilter ref="A2:I10" xr:uid="{DE7A74B4-1B1A-41BC-BD71-6686D3A80317}"/>
   <tableColumns count="9">
     <tableColumn id="1" xr3:uid="{AEDCF761-C41E-45F9-8585-F195D983B89C}" name="Nummer" dataDxfId="21"/>
     <tableColumn id="2" xr3:uid="{635CD206-F27E-4A6A-BC65-EEED36933D1E}" name="Naam" dataDxfId="20"/>
@@ -2434,7 +2440,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7034CDAF-2A08-4BE8-92C3-F4E7A6F24E1B}">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I10"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="13.28515625" style="18" customWidth="1"/>
@@ -2500,8 +2506,8 @@
         <v>57</v>
       </c>
       <c r="H3" s="28"/>
-      <c r="I3" s="29" t="b">
-        <f t="shared" ref="I3:I12" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
+      <c r="I3" s="18" t="b">
+        <f t="shared" ref="I3:I10" si="0">ISNUMBER(SEARCH("EHDS", G3))</f>
         <v>1</v>
       </c>
     </row>
@@ -2524,7 +2530,7 @@
       <c r="G4" s="18" t="s">
         <v>60</v>
       </c>
-      <c r="I4" s="29" t="b">
+      <c r="I4" s="18" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2551,7 +2557,7 @@
       <c r="H5" s="18" t="s">
         <v>65</v>
       </c>
-      <c r="I5" s="29" t="b">
+      <c r="I5" s="18" t="b">
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
@@ -2572,154 +2578,115 @@
       <c r="E6" s="18" t="s">
         <v>56</v>
       </c>
-      <c r="G6" s="30" t="s">
+      <c r="G6" s="29" t="s">
         <v>57</v>
       </c>
-      <c r="I6" s="29" t="b">
+      <c r="I6" s="18" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:9" ht="16.5" customHeight="1">
+    <row r="7" spans="1:9" ht="39" customHeight="1">
+      <c r="A7" s="18" t="s">
+        <v>69</v>
+      </c>
       <c r="B7" s="18" t="s">
-        <v>69</v>
+        <v>70</v>
+      </c>
+      <c r="C7" s="18" t="s">
+        <v>71</v>
       </c>
       <c r="D7" s="18" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="E7" s="18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G7" s="18" t="s">
-        <v>41</v>
-      </c>
-      <c r="I7" s="29" t="b">
-        <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:9" ht="39" customHeight="1">
-      <c r="A8" s="18" t="s">
-        <v>72</v>
-      </c>
-      <c r="B8" s="18" t="s">
-        <v>73</v>
-      </c>
-      <c r="C8" s="18" t="s">
         <v>74</v>
       </c>
-      <c r="D8" s="18" t="s">
+      <c r="H7" s="18" t="s">
         <v>75</v>
       </c>
-      <c r="E8" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>76</v>
-      </c>
-      <c r="H8" s="18" t="s">
-        <v>77</v>
-      </c>
-      <c r="I8" s="29" t="b">
+      <c r="I7" s="18" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:9" ht="39" customHeight="1">
+    <row r="8" spans="1:9" ht="43.5">
+      <c r="A8" s="18" t="s">
+        <v>76</v>
+      </c>
+      <c r="B8" s="18" t="s">
+        <v>77</v>
+      </c>
+      <c r="C8" s="18" t="s">
+        <v>78</v>
+      </c>
+      <c r="D8" s="18" t="s">
+        <v>79</v>
+      </c>
+      <c r="E8" s="18" t="s">
+        <v>73</v>
+      </c>
+      <c r="G8" s="18" t="s">
+        <v>80</v>
+      </c>
+      <c r="H8" s="18" t="s">
+        <v>81</v>
+      </c>
+      <c r="I8" s="18" t="b">
+        <f t="shared" si="0"/>
+        <v>1</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="43.5">
+      <c r="A9" s="18" t="s">
+        <v>82</v>
+      </c>
       <c r="B9" s="18" t="s">
-        <v>73</v>
+        <v>83</v>
+      </c>
+      <c r="C9" s="18" t="s">
+        <v>84</v>
       </c>
       <c r="D9" s="18" t="s">
-        <v>75</v>
+        <v>85</v>
       </c>
       <c r="E9" s="18" t="s">
         <v>56</v>
       </c>
       <c r="G9" s="18" t="s">
-        <v>41</v>
+        <v>86</v>
       </c>
       <c r="H9" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="I9" s="29" t="b">
+        <v>81</v>
+      </c>
+      <c r="I9" s="18" t="b">
         <f t="shared" si="0"/>
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="10" spans="1:9" ht="43.5">
       <c r="A10" s="18" t="s">
-        <v>79</v>
+        <v>87</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>80</v>
+        <v>88</v>
       </c>
       <c r="C10" s="18" t="s">
-        <v>81</v>
+        <v>89</v>
       </c>
       <c r="D10" s="18" t="s">
-        <v>82</v>
+        <v>90</v>
       </c>
       <c r="E10" s="18" t="s">
-        <v>71</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="H10" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="I10" s="29" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="11" spans="1:9" ht="43.5">
-      <c r="A11" s="18" t="s">
-        <v>84</v>
-      </c>
-      <c r="B11" s="18" t="s">
-        <v>85</v>
-      </c>
-      <c r="C11" s="18" t="s">
-        <v>86</v>
-      </c>
-      <c r="D11" s="18" t="s">
-        <v>87</v>
-      </c>
-      <c r="E11" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="G11" s="18" t="s">
-        <v>83</v>
-      </c>
-      <c r="H11" s="18" t="s">
-        <v>78</v>
-      </c>
-      <c r="I11" s="29" t="b">
-        <f t="shared" si="0"/>
-        <v>1</v>
-      </c>
-    </row>
-    <row r="12" spans="1:9" ht="43.5">
-      <c r="A12" s="18" t="s">
-        <v>88</v>
-      </c>
-      <c r="B12" s="18" t="s">
-        <v>89</v>
-      </c>
-      <c r="C12" s="18" t="s">
-        <v>90</v>
-      </c>
-      <c r="D12" s="18" t="s">
         <v>91</v>
       </c>
-      <c r="E12" s="18" t="s">
-        <v>92</v>
-      </c>
-      <c r="G12" s="30" t="s">
-        <v>57</v>
-      </c>
-      <c r="I12" s="29" t="b">
+      <c r="G10" s="29" t="s">
+        <v>74</v>
+      </c>
+      <c r="I10" s="18" t="b">
         <f t="shared" si="0"/>
         <v>1</v>
       </c>
@@ -2751,10 +2718,10 @@
   <sheetData>
     <row r="1" spans="1:7" ht="195.75" customHeight="1">
       <c r="A1" s="2" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="2" t="s">
         <v>93</v>
-      </c>
-      <c r="B1" s="2" t="s">
-        <v>94</v>
       </c>
       <c r="C1" s="2" t="s">
         <v>44</v>
@@ -2774,25 +2741,25 @@
     </row>
     <row r="2" spans="1:7">
       <c r="A2" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="B2" s="1" t="s">
         <v>95</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="C2" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="D2" s="1" t="s">
         <v>97</v>
       </c>
-      <c r="D2" s="1" t="s">
+      <c r="E2" s="1" t="s">
         <v>98</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="F2" s="1" t="s">
         <v>99</v>
       </c>
-      <c r="F2" s="1" t="s">
+      <c r="G2" s="1" t="s">
         <v>100</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>101</v>
       </c>
     </row>
   </sheetData>
@@ -2815,48 +2782,48 @@
     <row r="1" spans="1:4" ht="111" customHeight="1"/>
     <row r="2" spans="1:4" ht="15">
       <c r="A2" s="21" t="s">
+        <v>101</v>
+      </c>
+      <c r="B2" s="22" t="s">
         <v>102</v>
       </c>
-      <c r="B2" s="22" t="s">
+      <c r="C2" s="22" t="s">
         <v>103</v>
       </c>
-      <c r="C2" s="22" t="s">
+      <c r="D2" s="23" t="s">
         <v>104</v>
-      </c>
-      <c r="D2" s="23" t="s">
-        <v>105</v>
       </c>
     </row>
     <row r="3" spans="1:4" ht="15">
       <c r="A3" s="24" t="s">
+        <v>105</v>
+      </c>
+      <c r="B3" s="25" t="s">
         <v>106</v>
       </c>
-      <c r="B3" s="25" t="s">
+      <c r="C3" s="25" t="s">
         <v>107</v>
-      </c>
-      <c r="C3" s="25" t="s">
-        <v>108</v>
       </c>
       <c r="D3" s="26"/>
     </row>
     <row r="4" spans="1:4" ht="29.25">
       <c r="A4" s="24" t="s">
+        <v>108</v>
+      </c>
+      <c r="B4" s="25" t="s">
+        <v>106</v>
+      </c>
+      <c r="C4" s="25" t="s">
         <v>109</v>
-      </c>
-      <c r="B4" s="25" t="s">
-        <v>107</v>
-      </c>
-      <c r="C4" s="25" t="s">
-        <v>110</v>
       </c>
       <c r="D4" s="26"/>
     </row>
     <row r="5" spans="1:4" ht="15">
       <c r="A5" t="s">
+        <v>110</v>
+      </c>
+      <c r="C5" t="s">
         <v>111</v>
-      </c>
-      <c r="C5" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="6" spans="1:4" ht="15"/>
@@ -2888,7 +2855,7 @@
     <row r="2" spans="1:9">
       <c r="A2" s="4"/>
       <c r="B2" s="9" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C2" s="6"/>
       <c r="D2" s="6"/>
@@ -2901,16 +2868,16 @@
     <row r="3" spans="1:9" ht="29.25">
       <c r="A3" s="4"/>
       <c r="B3" s="8" t="s">
+        <v>101</v>
+      </c>
+      <c r="C3" s="8" t="s">
         <v>102</v>
       </c>
-      <c r="C3" s="8" t="s">
+      <c r="D3" s="8" t="s">
         <v>103</v>
       </c>
-      <c r="D3" s="8" t="s">
+      <c r="E3" s="10" t="s">
         <v>104</v>
-      </c>
-      <c r="E3" s="10" t="s">
-        <v>105</v>
       </c>
       <c r="F3" s="16" t="s">
         <v>50</v>
@@ -2922,16 +2889,16 @@
     <row r="4" spans="1:9" ht="48.75" customHeight="1">
       <c r="A4" s="4"/>
       <c r="B4" s="6" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C4" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D4" s="6" t="s">
         <v>114</v>
       </c>
-      <c r="D4" s="6" t="s">
+      <c r="E4" s="6" t="s">
         <v>115</v>
-      </c>
-      <c r="E4" s="6" t="s">
-        <v>116</v>
       </c>
       <c r="F4" s="6"/>
       <c r="G4" s="4"/>
@@ -2940,154 +2907,164 @@
     </row>
     <row r="5" spans="1:9" ht="43.5">
       <c r="B5" s="6" t="s">
+        <v>116</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D5" s="6" t="s">
         <v>117</v>
       </c>
-      <c r="C5" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D5" s="6" t="s">
+      <c r="E5" s="6" t="s">
         <v>118</v>
-      </c>
-      <c r="E5" s="6" t="s">
-        <v>119</v>
       </c>
       <c r="F5" s="6"/>
     </row>
     <row r="6" spans="1:9" ht="29.25">
       <c r="B6" s="6" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C6" s="6"/>
       <c r="D6" s="6" t="s">
+        <v>120</v>
+      </c>
+      <c r="E6" s="6" t="s">
         <v>121</v>
-      </c>
-      <c r="E6" s="6" t="s">
-        <v>122</v>
       </c>
       <c r="F6" s="6"/>
     </row>
     <row r="7" spans="1:9" ht="30.75" customHeight="1">
       <c r="B7" s="6" t="s">
+        <v>122</v>
+      </c>
+      <c r="C7" s="6" t="s">
+        <v>113</v>
+      </c>
+      <c r="D7" s="6" t="s">
         <v>123</v>
       </c>
-      <c r="C7" s="6" t="s">
-        <v>114</v>
-      </c>
-      <c r="D7" s="6" t="s">
+      <c r="E7" s="6" t="s">
         <v>124</v>
-      </c>
-      <c r="E7" s="6" t="s">
-        <v>125</v>
       </c>
       <c r="F7" s="6"/>
     </row>
     <row r="8" spans="1:9" ht="29.25">
       <c r="B8" s="6" t="s">
+        <v>125</v>
+      </c>
+      <c r="C8" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D8" s="6" t="s">
         <v>126</v>
       </c>
-      <c r="C8" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D8" s="6" t="s">
+      <c r="E8" s="6" t="s">
         <v>127</v>
       </c>
-      <c r="E8" s="6" t="s">
+      <c r="F8" s="6" t="s">
         <v>128</v>
-      </c>
-      <c r="F8" s="6" t="s">
-        <v>129</v>
       </c>
     </row>
     <row r="9" spans="1:9" ht="15">
       <c r="B9" s="6" t="s">
+        <v>105</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>106</v>
       </c>
-      <c r="C9" s="6" t="s">
+      <c r="D9" s="6" t="s">
         <v>107</v>
       </c>
-      <c r="D9" s="6" t="s">
-        <v>108</v>
-      </c>
       <c r="E9" s="6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="F9" s="6"/>
     </row>
     <row r="10" spans="1:9" ht="29.25">
       <c r="B10" s="6" t="s">
+        <v>108</v>
+      </c>
+      <c r="C10" s="6" t="s">
+        <v>106</v>
+      </c>
+      <c r="D10" s="6" t="s">
         <v>109</v>
       </c>
-      <c r="C10" s="6" t="s">
-        <v>107</v>
-      </c>
-      <c r="D10" s="6" t="s">
-        <v>110</v>
-      </c>
       <c r="E10" s="6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="F10" s="6"/>
     </row>
     <row r="11" spans="1:9" ht="15">
       <c r="B11" s="14" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C11" s="6"/>
       <c r="D11" s="6" t="s">
+        <v>132</v>
+      </c>
+      <c r="E11" s="6" t="s">
         <v>133</v>
-      </c>
-      <c r="E11" s="6" t="s">
-        <v>134</v>
       </c>
       <c r="F11" s="6"/>
     </row>
     <row r="12" spans="1:9" ht="29.25">
       <c r="B12" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C12" s="6" t="s">
         <v>135</v>
       </c>
-      <c r="C12" s="6" t="s">
+      <c r="D12" s="6" t="s">
         <v>136</v>
-      </c>
-      <c r="D12" s="6" t="s">
-        <v>137</v>
       </c>
       <c r="E12" s="6"/>
       <c r="F12" s="6" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="13" spans="1:9" ht="15">
       <c r="B13" s="6" t="s">
+        <v>138</v>
+      </c>
+      <c r="C13" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D13" t="s">
         <v>139</v>
-      </c>
-      <c r="C13" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D13" t="s">
-        <v>140</v>
       </c>
       <c r="E13" s="6"/>
       <c r="F13" s="6"/>
     </row>
     <row r="14" spans="1:9" ht="15">
       <c r="B14" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="C14" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="D14" t="s">
         <v>141</v>
-      </c>
-      <c r="C14" s="6" t="s">
-        <v>136</v>
-      </c>
-      <c r="D14" t="s">
-        <v>142</v>
       </c>
       <c r="E14" s="6"/>
       <c r="F14" s="6"/>
     </row>
     <row r="15" spans="1:9" ht="15">
-      <c r="B15" s="6"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
+      <c r="B15" s="6" t="s">
+        <v>134</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>144</v>
+      </c>
+      <c r="F15" s="6" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="16" spans="1:9" ht="15">
       <c r="B16" s="6"/>
@@ -3137,6 +3114,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100D5656983173B1142A9B62A9C329F89A7" ma:contentTypeVersion="13" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="71caa5f225d89a4181f0614974a0635b">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="bb18a1b9-ddba-4244-9634-64732d0cb267" xmlns:ns3="06294a2e-6f87-4144-83b8-94a4d04d144a" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="d74eef483bec37fcdf125766e7bdb283" ns2:_="" ns3:_="">
     <xsd:import namespace="bb18a1b9-ddba-4244-9634-64732d0cb267"/>
@@ -3343,15 +3329,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -3364,11 +3341,11 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{148267B0-4CF5-48A7-B543-CDE45AF0A8FC}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{14B9AD58-A794-48C7-986D-80A9DB4B3205}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>

</xml_diff>